<commit_message>
feat: expand valuation comparables
</commit_message>
<xml_diff>
--- a/model/valuation_model.xlsx
+++ b/model/valuation_model.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="Re197d42b2781491d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bear" sheetId="2" r:id="Rd2b29aba89324afa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="3" r:id="Rd690e2045c7b44fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull" sheetId="4" r:id="Rb87c17f8d2454350"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="Rd4b4107e20784476"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="6" r:id="Rc5a7e46d235946a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="R0911522af87246f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bear" sheetId="2" r:id="R846cb796213d4f1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="3" r:id="Re41f25e0c8b64d01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull" sheetId="4" r:id="Re441402e73af473d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="R2ff0769751fc4b31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="6" r:id="Ra2e1c53892de4656"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Comps" sheetId="7" r:id="R9b422fcb576a4184"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +19,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="2">
+  <x:numFmts count="3">
+    <x:numFmt numFmtId="200" formatCode="0.000"/>
+    <x:numFmt numFmtId="201" formatCode="0"/>
+    <x:numFmt numFmtId="202" formatCode="0.0&quot;x&quot;"/>
+  </x:numFmts>
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -27,8 +33,25 @@
     <x:font>
       <x:b/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF222222"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFC62828"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -40,17 +63,403 @@
         <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE8E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDEBF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7E6E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE8E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDEBF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7E6E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="3">
     <x:border/>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFB4C6E7"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFB4C6E7"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFB4C6E7"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB4C6E7"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="3">
+  <x:cellXfs count="109">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="2" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -342,9 +751,9 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16" customWidth="1"/>
-    <x:col min="2" max="2" width="16" customWidth="1"/>
-    <x:col min="3" max="3" width="16" customWidth="1"/>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="72" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -2846,10 +3255,10 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16" customWidth="1"/>
-    <x:col min="2" max="2" width="16" customWidth="1"/>
-    <x:col min="3" max="3" width="16" customWidth="1"/>
-    <x:col min="4" max="4" width="16" customWidth="1"/>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -2992,8 +3401,8 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16" customWidth="1"/>
-    <x:col min="2" max="2" width="16" customWidth="1"/>
+    <x:col min="1" max="1" width="42" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -3027,10 +3436,8 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Market EV / FY2026E revenue</x:t>
-        </x:is>
+      <x:c r="A4" t="str">
+        <x:v>Market equity value / FY2026E revenue</x:v>
       </x:c>
       <x:c r="B4" t="n">
         <x:v>311.5</x:v>
@@ -3094,6 +3501,573 @@
       </x:c>
       <x:c r="B10" t="n">
         <x:v>0.0298</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF1F4E78"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="27" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="10" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="27" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="38" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="38" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="52" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="63" t="str">
+        <x:v>company</x:v>
+      </x:c>
+      <x:c r="B1" s="63" t="str">
+        <x:v>ticker</x:v>
+      </x:c>
+      <x:c r="C1" s="63" t="str">
+        <x:v>cohort</x:v>
+      </x:c>
+      <x:c r="D1" s="63" t="str">
+        <x:v>valuation_date</x:v>
+      </x:c>
+      <x:c r="E1" s="63" t="str">
+        <x:v>valuation_basis</x:v>
+      </x:c>
+      <x:c r="F1" s="63" t="str">
+        <x:v>equity_value_bn</x:v>
+      </x:c>
+      <x:c r="G1" s="63" t="str">
+        <x:v>revenue_bn</x:v>
+      </x:c>
+      <x:c r="H1" s="63" t="str">
+        <x:v>currency</x:v>
+      </x:c>
+      <x:c r="I1" s="63" t="str">
+        <x:v>revenue_basis</x:v>
+      </x:c>
+      <x:c r="J1" s="63" t="str">
+        <x:v>include_in_private_range</x:v>
+      </x:c>
+      <x:c r="K1" s="63" t="str">
+        <x:v>valuation_source_url</x:v>
+      </x:c>
+      <x:c r="L1" s="63" t="str">
+        <x:v>revenue_source_url</x:v>
+      </x:c>
+      <x:c r="M1" s="63" t="str">
+        <x:v>comparability_note</x:v>
+      </x:c>
+      <x:c r="N1" s="63" t="str">
+        <x:v>multiple_x</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="46" customHeight="1">
+      <x:c r="A2" s="65" t="str">
+        <x:v>Zhipu</x:v>
+      </x:c>
+      <x:c r="B2" s="65" t="str">
+        <x:v>02513.HK</x:v>
+      </x:c>
+      <x:c r="C2" s="65" t="str">
+        <x:v>core_frontier</x:v>
+      </x:c>
+      <x:c r="D2" s="81" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="E2" s="101" t="str">
+        <x:v>public market equity value</x:v>
+      </x:c>
+      <x:c r="F2" s="85" t="str">
+        <x:v>62.303701</x:v>
+      </x:c>
+      <x:c r="G2" s="85" t="str">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="H2" s="86" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I2" s="105" t="str">
+        <x:v>FY2026E model revenue</x:v>
+      </x:c>
+      <x:c r="J2" s="87" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K2" s="101" t="str">
+        <x:v>https://tushare.pro/document/2?doc_id=192</x:v>
+      </x:c>
+      <x:c r="L2" s="101" t="str">
+        <x:v>https://github.com/ericxuzhesheng/Zhipu-AI-Valuation/blob/main/model/valuation_model.xlsx</x:v>
+      </x:c>
+      <x:c r="M2" s="101" t="str">
+        <x:v>Subject company; equity value and revenue are refreshed from the local market file and model assumptions.</x:v>
+      </x:c>
+      <x:c r="N2" s="97" t="n">
+        <x:f>F2/G2</x:f>
+        <x:v>311.51850499999995</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="46" customHeight="1">
+      <x:c r="A3" s="66" t="str">
+        <x:v>MiniMax</x:v>
+      </x:c>
+      <x:c r="B3" s="66" t="str">
+        <x:v>00100.HK</x:v>
+      </x:c>
+      <x:c r="C3" s="66" t="str">
+        <x:v>core_frontier</x:v>
+      </x:c>
+      <x:c r="D3" s="82" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="E3" s="102" t="str">
+        <x:v>public market equity value</x:v>
+      </x:c>
+      <x:c r="F3" s="88" t="str">
+        <x:v>13.450037</x:v>
+      </x:c>
+      <x:c r="G3" s="88" t="str">
+        <x:v>0.165182</x:v>
+      </x:c>
+      <x:c r="H3" s="89" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I3" s="106" t="str">
+        <x:v>LTM through 2026H1</x:v>
+      </x:c>
+      <x:c r="J3" s="90" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K3" s="102" t="str">
+        <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0806/2026080601088.pdf</x:v>
+      </x:c>
+      <x:c r="L3" s="102" t="str">
+        <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0826/2026082600680.pdf</x:v>
+      </x:c>
+      <x:c r="M3" s="102" t="str">
+        <x:v>Closest listed foundation-model peer; public-market LTM multiple is shown separately from private transaction references.</x:v>
+      </x:c>
+      <x:c r="N3" s="98" t="n">
+        <x:f>F3/G3</x:f>
+        <x:v>81.42556089646573</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="46" customHeight="1">
+      <x:c r="A4" s="66" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="B4" s="66" t="str">
+        <x:v>private</x:v>
+      </x:c>
+      <x:c r="C4" s="66" t="str">
+        <x:v>core_frontier</x:v>
+      </x:c>
+      <x:c r="D4" s="82" t="str">
+        <x:v>2026-03-31</x:v>
+      </x:c>
+      <x:c r="E4" s="102" t="str">
+        <x:v>post-money financing</x:v>
+      </x:c>
+      <x:c r="F4" s="88" t="str">
+        <x:v>852.0</x:v>
+      </x:c>
+      <x:c r="G4" s="88" t="str">
+        <x:v>25.0</x:v>
+      </x:c>
+      <x:c r="H4" s="89" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I4" s="106" t="str">
+        <x:v>annualized revenue at February 2026</x:v>
+      </x:c>
+      <x:c r="J4" s="90" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K4" s="102" t="str">
+        <x:v>https://openai.com/index/accelerating-the-next-phase-ai/</x:v>
+      </x:c>
+      <x:c r="L4" s="102" t="str">
+        <x:v>https://finance.yahoo.com/news/openai-tops-25-billion-annualized-033836274.html</x:v>
+      </x:c>
+      <x:c r="M4" s="102" t="str">
+        <x:v>Private frontier-lab transaction reference; revenue was reported by Reuters and was not independently verified.</x:v>
+      </x:c>
+      <x:c r="N4" s="98" t="n">
+        <x:f>F4/G4</x:f>
+        <x:v>34.08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="46" customHeight="1">
+      <x:c r="A5" s="66" t="str">
+        <x:v>Anthropic</x:v>
+      </x:c>
+      <x:c r="B5" s="66" t="str">
+        <x:v>private</x:v>
+      </x:c>
+      <x:c r="C5" s="66" t="str">
+        <x:v>core_frontier</x:v>
+      </x:c>
+      <x:c r="D5" s="82" t="str">
+        <x:v>2026-05-28</x:v>
+      </x:c>
+      <x:c r="E5" s="102" t="str">
+        <x:v>post-money financing</x:v>
+      </x:c>
+      <x:c r="F5" s="88" t="str">
+        <x:v>965.0</x:v>
+      </x:c>
+      <x:c r="G5" s="88" t="str">
+        <x:v>47.0</x:v>
+      </x:c>
+      <x:c r="H5" s="89" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I5" s="106" t="str">
+        <x:v>annualized revenue at May 2026</x:v>
+      </x:c>
+      <x:c r="J5" s="90" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K5" s="102" t="str">
+        <x:v>https://www.anthropic.com/news/series-h</x:v>
+      </x:c>
+      <x:c r="L5" s="102" t="str">
+        <x:v>https://www.anthropic.com/news/series-h</x:v>
+      </x:c>
+      <x:c r="M5" s="102" t="str">
+        <x:v>Private frontier-lab transaction reference with valuation and revenue disclosed together by the company.</x:v>
+      </x:c>
+      <x:c r="N5" s="98" t="n">
+        <x:f>F5/G5</x:f>
+        <x:v>20.53191489361702</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="46" customHeight="1">
+      <x:c r="A6" s="66" t="str">
+        <x:v>Mistral</x:v>
+      </x:c>
+      <x:c r="B6" s="66" t="str">
+        <x:v>private</x:v>
+      </x:c>
+      <x:c r="C6" s="66" t="str">
+        <x:v>core_frontier</x:v>
+      </x:c>
+      <x:c r="D6" s="82" t="str">
+        <x:v>2025-09-09</x:v>
+      </x:c>
+      <x:c r="E6" s="102" t="str">
+        <x:v>post-money financing</x:v>
+      </x:c>
+      <x:c r="F6" s="88" t="str">
+        <x:v>11.7</x:v>
+      </x:c>
+      <x:c r="G6" s="88" t="str">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="H6" s="89" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I6" s="106" t="str">
+        <x:v>annualized revenue at September 2025</x:v>
+      </x:c>
+      <x:c r="J6" s="90" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K6" s="102" t="str">
+        <x:v>https://mistral.ai/news/mistral-ai-raises-1-7-b-to-accelerate-technological-progress-with-ai/</x:v>
+      </x:c>
+      <x:c r="L6" s="102" t="str">
+        <x:v>https://www.lemonde.fr/economie/article/2025/09/26/mistral-ai-incarnation-de-l-intelligence-artificielle_6643087_3234.html</x:v>
+      </x:c>
+      <x:c r="M6" s="102" t="str">
+        <x:v>Older private frontier-lab reference; included in the private transaction range but dated separately.</x:v>
+      </x:c>
+      <x:c r="N6" s="98" t="n">
+        <x:f>F6/G6</x:f>
+        <x:v>39</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="46" customHeight="1">
+      <x:c r="A7" s="67" t="str">
+        <x:v>SenseTime</x:v>
+      </x:c>
+      <x:c r="B7" s="67" t="str">
+        <x:v>00020.HK</x:v>
+      </x:c>
+      <x:c r="C7" s="67" t="str">
+        <x:v>hk_adjacent</x:v>
+      </x:c>
+      <x:c r="D7" s="83" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="E7" s="103" t="str">
+        <x:v>implied total equity value</x:v>
+      </x:c>
+      <x:c r="F7" s="91" t="str">
+        <x:v>54.04443</x:v>
+      </x:c>
+      <x:c r="G7" s="91" t="str">
+        <x:v>5.567388</x:v>
+      </x:c>
+      <x:c r="H7" s="92" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="I7" s="107" t="str">
+        <x:v>LTM through 2026H1</x:v>
+      </x:c>
+      <x:c r="J7" s="93" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K7" s="103" t="str">
+        <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0805/2026080500774.pdf</x:v>
+      </x:c>
+      <x:c r="L7" s="103" t="str">
+        <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0826/2026082600408.pdf</x:v>
+      </x:c>
+      <x:c r="M7" s="103" t="str">
+        <x:v>Adjacent Hong Kong AI platform; mixed computer-vision generative-AI and solution revenue makes it contextual only.</x:v>
+      </x:c>
+      <x:c r="N7" s="99" t="n">
+        <x:f>F7/G7</x:f>
+        <x:v>9.70732235655212</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="46" customHeight="1">
+      <x:c r="A8" s="67" t="str">
+        <x:v>Phancy</x:v>
+      </x:c>
+      <x:c r="B8" s="67" t="str">
+        <x:v>06682.HK</x:v>
+      </x:c>
+      <x:c r="C8" s="67" t="str">
+        <x:v>hk_adjacent</x:v>
+      </x:c>
+      <x:c r="D8" s="83" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="E8" s="103" t="str">
+        <x:v>implied total equity value</x:v>
+      </x:c>
+      <x:c r="F8" s="91" t="str">
+        <x:v>13.375496</x:v>
+      </x:c>
+      <x:c r="G8" s="91" t="str">
+        <x:v>8.274083</x:v>
+      </x:c>
+      <x:c r="H8" s="92" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="I8" s="107" t="str">
+        <x:v>LTM through 2026H1</x:v>
+      </x:c>
+      <x:c r="J8" s="93" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K8" s="103" t="str">
+        <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0805/2026080500986.pdf</x:v>
+      </x:c>
+      <x:c r="L8" s="103" t="str">
+        <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0820/2026082000357.pdf</x:v>
+      </x:c>
+      <x:c r="M8" s="103" t="str">
+        <x:v>Enterprise AI platform and agentic services with a different revenue and margin mix; contextual only.</x:v>
+      </x:c>
+      <x:c r="N8" s="99" t="n">
+        <x:f>F8/G8</x:f>
+        <x:v>1.6165532784720678</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="46" customHeight="1">
+      <x:c r="A9" s="67" t="str">
+        <x:v>Wenge AI</x:v>
+      </x:c>
+      <x:c r="B9" s="67" t="str">
+        <x:v>01956.HK</x:v>
+      </x:c>
+      <x:c r="C9" s="67" t="str">
+        <x:v>hk_adjacent</x:v>
+      </x:c>
+      <x:c r="D9" s="83" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="E9" s="103" t="str">
+        <x:v>implied total equity value</x:v>
+      </x:c>
+      <x:c r="F9" s="91" t="str">
+        <x:v>13.240056</x:v>
+      </x:c>
+      <x:c r="G9" s="91" t="str">
+        <x:v>0.459773</x:v>
+      </x:c>
+      <x:c r="H9" s="92" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="I9" s="107" t="str">
+        <x:v>LTM through 2026H1</x:v>
+      </x:c>
+      <x:c r="J9" s="93" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K9" s="103" t="str">
+        <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0805/2026080501012.pdf</x:v>
+      </x:c>
+      <x:c r="L9" s="103" t="str">
+        <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0825/2026082500959.pdf</x:v>
+      </x:c>
+      <x:c r="M9" s="103" t="str">
+        <x:v>Decision-intelligence and project-delivery model with a short trading history; contextual only.</x:v>
+      </x:c>
+      <x:c r="N9" s="99" t="n">
+        <x:f>F9/G9</x:f>
+        <x:v>28.7969410991946</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="46" customHeight="1">
+      <x:c r="A10" s="68" t="str">
+        <x:v>Palantir</x:v>
+      </x:c>
+      <x:c r="B10" s="68" t="str">
+        <x:v>PLTR</x:v>
+      </x:c>
+      <x:c r="C10" s="68" t="str">
+        <x:v>commercialization_reference</x:v>
+      </x:c>
+      <x:c r="D10" s="84" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="E10" s="104" t="str">
+        <x:v>public market equity value</x:v>
+      </x:c>
+      <x:c r="F10" s="94" t="str">
+        <x:v>447.64</x:v>
+      </x:c>
+      <x:c r="G10" s="94" t="str">
+        <x:v>4.475446</x:v>
+      </x:c>
+      <x:c r="H10" s="95" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I10" s="108" t="str">
+        <x:v>FY2025 revenue</x:v>
+      </x:c>
+      <x:c r="J10" s="96" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K10" s="104" t="str">
+        <x:v>https://www.gurufocus.com/stock/PLTR/data/market-cap</x:v>
+      </x:c>
+      <x:c r="L10" s="104" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1321655/000132165526000011/pltr-20251231.htm</x:v>
+      </x:c>
+      <x:c r="M10" s="104" t="str">
+        <x:v>Mature AI software commercialization reference; not a frontier-model laboratory.</x:v>
+      </x:c>
+      <x:c r="N10" s="100" t="n">
+        <x:f>F10/G10</x:f>
+        <x:v>100.0213163112682</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="46" customHeight="1">
+      <x:c r="A11" s="68" t="str">
+        <x:v>Cloudflare</x:v>
+      </x:c>
+      <x:c r="B11" s="68" t="str">
+        <x:v>NET</x:v>
+      </x:c>
+      <x:c r="C11" s="68" t="str">
+        <x:v>commercialization_reference</x:v>
+      </x:c>
+      <x:c r="D11" s="84" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="E11" s="104" t="str">
+        <x:v>public market equity value</x:v>
+      </x:c>
+      <x:c r="F11" s="94" t="str">
+        <x:v>106.39</x:v>
+      </x:c>
+      <x:c r="G11" s="94" t="str">
+        <x:v>2.1679</x:v>
+      </x:c>
+      <x:c r="H11" s="95" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I11" s="108" t="str">
+        <x:v>FY2025 revenue</x:v>
+      </x:c>
+      <x:c r="J11" s="96" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K11" s="104" t="str">
+        <x:v>https://www.tipranks.com/stocks/net/market-cap</x:v>
+      </x:c>
+      <x:c r="L11" s="104" t="str">
+        <x:v>https://www.cloudflare.com/press/press-releases/2026/cloudflare-announces-fourth-quarter-and-fiscal-year-2025-financial-results/</x:v>
+      </x:c>
+      <x:c r="M11" s="104" t="str">
+        <x:v>Connectivity and inference-infrastructure reference; economics differ from a model laboratory.</x:v>
+      </x:c>
+      <x:c r="N11" s="100" t="n">
+        <x:f>F11/G11</x:f>
+        <x:v>49.0751418423359</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="46" customHeight="1">
+      <x:c r="A12" s="68" t="str">
+        <x:v>Snowflake</x:v>
+      </x:c>
+      <x:c r="B12" s="68" t="str">
+        <x:v>SNOW</x:v>
+      </x:c>
+      <x:c r="C12" s="68" t="str">
+        <x:v>commercialization_reference</x:v>
+      </x:c>
+      <x:c r="D12" s="84" t="str">
+        <x:v>2026-08-28</x:v>
+      </x:c>
+      <x:c r="E12" s="104" t="str">
+        <x:v>public market equity value</x:v>
+      </x:c>
+      <x:c r="F12" s="94" t="str">
+        <x:v>113.685</x:v>
+      </x:c>
+      <x:c r="G12" s="94" t="str">
+        <x:v>4.683946</x:v>
+      </x:c>
+      <x:c r="H12" s="95" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I12" s="108" t="str">
+        <x:v>FY2026 revenue</x:v>
+      </x:c>
+      <x:c r="J12" s="96" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K12" s="104" t="str">
+        <x:v>https://finance.yahoo.com/quote/SNOW/</x:v>
+      </x:c>
+      <x:c r="L12" s="104" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1640147/000164014726000023/snowflake2026ars.pdf</x:v>
+      </x:c>
+      <x:c r="M12" s="104" t="str">
+        <x:v>Data-cloud commercialization reference; not a direct foundation-model comparable.</x:v>
+      </x:c>
+      <x:c r="N12" s="100" t="n">
+        <x:f>F12/G12</x:f>
+        <x:v>24.271202101817572</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Standardize listed peer multiples on LTM revenue
</commit_message>
<xml_diff>
--- a/model/valuation_model.xlsx
+++ b/model/valuation_model.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="R9f3e8c091f774283"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bear" sheetId="2" r:id="R2b9690ca93574edc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="3" r:id="Rdf23ff86ba1b4a7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull" sheetId="4" r:id="Rce38106d405044e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="R1fe4655150494bd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Comps" sheetId="6" r:id="R94a377fc69c7414a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="7" r:id="R13ab7e9d98d74fae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="Rc240d3ab765242df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bear" sheetId="2" r:id="R09f01bfdb4954575"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="3" r:id="R42ed4a9da89b4c29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull" sheetId="4" r:id="Rc3b6c825c8f0487d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="Rff5c854a24284c05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Comps" sheetId="6" r:id="Red3020c606e74f88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="7" r:id="R2372e65b90254933"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -63,7 +63,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -73,36 +73,6 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFD9EAF7"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF1F4E78"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFD9EAF7"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF2CC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFCE8E6"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFDDEBF7"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE7E6E6"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -184,7 +154,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="89">
+  <x:cellXfs count="59">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -344,96 +314,6 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="204" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="5" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="5" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="205" fontId="6" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="204" fontId="6" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="205" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="204" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="205" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="204" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="205" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="204" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -733,13 +613,13 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="59" t="inlineStr">
+      <x:c r="A1" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">GLOBAL ASSUMPTIONS</x:t>
         </x:is>
       </x:c>
-      <x:c r="B1" s="60"/>
-      <x:c r="C1" s="60"/>
+      <x:c r="B1" s="10"/>
+      <x:c r="C1" s="10"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="6" t="inlineStr">
@@ -868,133 +748,148 @@
     <x:row r="12">
       <x:c r="A12" s="6" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">2026H1 revenue (RMB m)</x:t>
+          <x:t xml:space="preserve">LTM revenue through 2026H1 (US$m)</x:t>
         </x:is>
       </x:c>
       <x:c r="B12" s="14" t="n">
-        <x:v>953.8920000000001</x:v>
+        <x:v>209.480985915493</x:v>
       </x:c>
       <x:c r="C12" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">unaudited; reviewed by KPMG</x:t>
+          <x:t xml:space="preserve">FY2025 less 2025H1 plus 2026H1, translated at USD/CNY 7.1</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="6" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">2026H1 total gross margin</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B13" s="12" t="n">
-        <x:v>0.2637730476825468</x:v>
-      </x:c>
-      <x:c r="C13" s="11"/>
+          <x:t xml:space="preserve">2026H1 revenue (RMB m)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" s="14" t="n">
+        <x:v>953.8920000000001</x:v>
+      </x:c>
+      <x:c r="C13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">unaudited; reviewed by KPMG</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="6" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">2026H1 API revenue share</x:t>
+          <x:t xml:space="preserve">2026H1 total gross margin</x:t>
         </x:is>
       </x:c>
       <x:c r="B14" s="12" t="n">
-        <x:v>0.8650622921672474</x:v>
+        <x:v>0.2637730476825468</x:v>
       </x:c>
       <x:c r="C14" s="11"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="6" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">2026H1 API gross margin</x:t>
+          <x:t xml:space="preserve">2026H1 API revenue share</x:t>
         </x:is>
       </x:c>
       <x:c r="B15" s="12" t="n">
-        <x:v>0.2458517940415136</x:v>
+        <x:v>0.8650622921672474</x:v>
       </x:c>
       <x:c r="C15" s="11"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="6" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">2026H1 operating margin</x:t>
+          <x:t xml:space="preserve">2026H1 API gross margin</x:t>
         </x:is>
       </x:c>
       <x:c r="B16" s="12" t="n">
-        <x:v>-2.250309259329148</x:v>
+        <x:v>0.2458517940415136</x:v>
       </x:c>
       <x:c r="C16" s="11"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="6" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">2026E operating margin</x:t>
+          <x:t xml:space="preserve">2026H1 operating margin</x:t>
         </x:is>
       </x:c>
       <x:c r="B17" s="12" t="n">
-        <x:v>-1</x:v>
-      </x:c>
-      <x:c r="C17" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">model assumption; H1 actual shown above</x:t>
-        </x:is>
-      </x:c>
+        <x:v>-2.250309259329148</x:v>
+      </x:c>
+      <x:c r="C17" s="11"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="6" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">2026H1 adjusted net loss (RMB m)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B18" s="14" t="n">
-        <x:v>1964.138</x:v>
-      </x:c>
-      <x:c r="C18" s="11"/>
+          <x:t xml:space="preserve">2026E operating margin</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" s="12" t="n">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="C18" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">model assumption; H1 actual shown above</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="6" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">2026-06-30 cash + ST investments (RMB m)</x:t>
+          <x:t xml:space="preserve">2026H1 adjusted net loss (RMB m)</x:t>
         </x:is>
       </x:c>
       <x:c r="B19" s="14" t="n">
-        <x:v>4499.861</x:v>
+        <x:v>1964.138</x:v>
       </x:c>
       <x:c r="C19" s="11"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="6" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">2026-06-30 bank loans + leases (RMB m)</x:t>
+          <x:t xml:space="preserve">2026-06-30 cash + ST investments (RMB m)</x:t>
         </x:is>
       </x:c>
       <x:c r="B20" s="14" t="n">
-        <x:v>2604.199</x:v>
+        <x:v>4499.861</x:v>
       </x:c>
       <x:c r="C20" s="11"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="6" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">2026-06-30 bank loans + leases (RMB m)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B21" s="14" t="n">
+        <x:v>2604.199</x:v>
+      </x:c>
+      <x:c r="C21" s="11"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="6" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve">July placement net proceeds (HKD m)</x:t>
         </x:is>
       </x:c>
-      <x:c r="B21" s="14" t="n">
+      <x:c r="B22" s="14" t="n">
         <x:v>31374.95</x:v>
       </x:c>
-      <x:c r="C21" s="11"/>
-    </x:row>
-    <x:row r="22" ht="36" customHeight="1">
-      <x:c r="A22" s="6" t="inlineStr">
+      <x:c r="C22" s="11"/>
+    </x:row>
+    <x:row r="23" ht="36" customHeight="1">
+      <x:c r="A23" s="6" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026H1 operating cash flow</x:t>
         </x:is>
       </x:c>
-      <x:c r="B22" s="6" t="inlineStr">
+      <x:c r="B23" s="6" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Not disclosed</x:t>
         </x:is>
       </x:c>
-      <x:c r="C22" s="11" t="inlineStr">
+      <x:c r="C23" s="11" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">interim results announcement did not include a cash-flow statement</x:t>
         </x:is>
@@ -1026,24 +921,24 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="62" t="inlineStr">
+      <x:c r="A1" s="20" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">DCF - Bear scenario</x:t>
         </x:is>
       </x:c>
-      <x:c r="B1" s="62"/>
-      <x:c r="C1" s="62"/>
-      <x:c r="D1" s="62"/>
-      <x:c r="E1" s="62"/>
-      <x:c r="F1" s="62"/>
-      <x:c r="G1" s="62"/>
-      <x:c r="H1" s="62"/>
-      <x:c r="I1" s="62"/>
-      <x:c r="J1" s="62"/>
-      <x:c r="K1" s="62"/>
-      <x:c r="L1" s="62"/>
-      <x:c r="M1" s="62"/>
-      <x:c r="N1" s="62"/>
+      <x:c r="B1" s="20"/>
+      <x:c r="C1" s="20"/>
+      <x:c r="D1" s="20"/>
+      <x:c r="E1" s="20"/>
+      <x:c r="F1" s="20"/>
+      <x:c r="G1" s="20"/>
+      <x:c r="H1" s="20"/>
+      <x:c r="I1" s="20"/>
+      <x:c r="J1" s="20"/>
+      <x:c r="K1" s="20"/>
+      <x:c r="L1" s="20"/>
+      <x:c r="M1" s="20"/>
+      <x:c r="N1" s="20"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="17" t="inlineStr">
@@ -1172,72 +1067,72 @@
       <x:c r="N7" s="17"/>
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
-      <x:c r="A8" s="63" t="inlineStr">
+      <x:c r="A8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Year</x:t>
         </x:is>
       </x:c>
-      <x:c r="B8" s="63" t="inlineStr">
+      <x:c r="B8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">i</x:t>
         </x:is>
       </x:c>
-      <x:c r="C8" s="63" t="inlineStr">
+      <x:c r="C8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">growth</x:t>
         </x:is>
       </x:c>
-      <x:c r="D8" s="63" t="inlineStr">
+      <x:c r="D8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">revenue</x:t>
         </x:is>
       </x:c>
-      <x:c r="E8" s="63" t="inlineStr">
+      <x:c r="E8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">op margin</x:t>
         </x:is>
       </x:c>
-      <x:c r="F8" s="63" t="inlineStr">
+      <x:c r="F8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">EBIT</x:t>
         </x:is>
       </x:c>
-      <x:c r="G8" s="63" t="inlineStr">
+      <x:c r="G8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">cash tax</x:t>
         </x:is>
       </x:c>
-      <x:c r="H8" s="63" t="inlineStr">
+      <x:c r="H8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">NOL end</x:t>
         </x:is>
       </x:c>
-      <x:c r="I8" s="63" t="inlineStr">
+      <x:c r="I8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">NOPAT</x:t>
         </x:is>
       </x:c>
-      <x:c r="J8" s="63" t="inlineStr">
+      <x:c r="J8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">dRev</x:t>
         </x:is>
       </x:c>
-      <x:c r="K8" s="63" t="inlineStr">
+      <x:c r="K8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">reinvest</x:t>
         </x:is>
       </x:c>
-      <x:c r="L8" s="63" t="inlineStr">
+      <x:c r="L8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">FCFF</x:t>
         </x:is>
       </x:c>
-      <x:c r="M8" s="63" t="inlineStr">
+      <x:c r="M8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">disc</x:t>
         </x:is>
       </x:c>
-      <x:c r="N8" s="63" t="inlineStr">
+      <x:c r="N8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">PV</x:t>
         </x:is>
@@ -2006,24 +1901,24 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="62" t="inlineStr">
+      <x:c r="A1" s="20" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">DCF - Base scenario</x:t>
         </x:is>
       </x:c>
-      <x:c r="B1" s="62"/>
-      <x:c r="C1" s="62"/>
-      <x:c r="D1" s="62"/>
-      <x:c r="E1" s="62"/>
-      <x:c r="F1" s="62"/>
-      <x:c r="G1" s="62"/>
-      <x:c r="H1" s="62"/>
-      <x:c r="I1" s="62"/>
-      <x:c r="J1" s="62"/>
-      <x:c r="K1" s="62"/>
-      <x:c r="L1" s="62"/>
-      <x:c r="M1" s="62"/>
-      <x:c r="N1" s="62"/>
+      <x:c r="B1" s="20"/>
+      <x:c r="C1" s="20"/>
+      <x:c r="D1" s="20"/>
+      <x:c r="E1" s="20"/>
+      <x:c r="F1" s="20"/>
+      <x:c r="G1" s="20"/>
+      <x:c r="H1" s="20"/>
+      <x:c r="I1" s="20"/>
+      <x:c r="J1" s="20"/>
+      <x:c r="K1" s="20"/>
+      <x:c r="L1" s="20"/>
+      <x:c r="M1" s="20"/>
+      <x:c r="N1" s="20"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="17" t="inlineStr">
@@ -2152,72 +2047,72 @@
       <x:c r="N7" s="17"/>
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
-      <x:c r="A8" s="63" t="inlineStr">
+      <x:c r="A8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Year</x:t>
         </x:is>
       </x:c>
-      <x:c r="B8" s="63" t="inlineStr">
+      <x:c r="B8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">i</x:t>
         </x:is>
       </x:c>
-      <x:c r="C8" s="63" t="inlineStr">
+      <x:c r="C8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">growth</x:t>
         </x:is>
       </x:c>
-      <x:c r="D8" s="63" t="inlineStr">
+      <x:c r="D8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">revenue</x:t>
         </x:is>
       </x:c>
-      <x:c r="E8" s="63" t="inlineStr">
+      <x:c r="E8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">op margin</x:t>
         </x:is>
       </x:c>
-      <x:c r="F8" s="63" t="inlineStr">
+      <x:c r="F8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">EBIT</x:t>
         </x:is>
       </x:c>
-      <x:c r="G8" s="63" t="inlineStr">
+      <x:c r="G8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">cash tax</x:t>
         </x:is>
       </x:c>
-      <x:c r="H8" s="63" t="inlineStr">
+      <x:c r="H8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">NOL end</x:t>
         </x:is>
       </x:c>
-      <x:c r="I8" s="63" t="inlineStr">
+      <x:c r="I8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">NOPAT</x:t>
         </x:is>
       </x:c>
-      <x:c r="J8" s="63" t="inlineStr">
+      <x:c r="J8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">dRev</x:t>
         </x:is>
       </x:c>
-      <x:c r="K8" s="63" t="inlineStr">
+      <x:c r="K8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">reinvest</x:t>
         </x:is>
       </x:c>
-      <x:c r="L8" s="63" t="inlineStr">
+      <x:c r="L8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">FCFF</x:t>
         </x:is>
       </x:c>
-      <x:c r="M8" s="63" t="inlineStr">
+      <x:c r="M8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">disc</x:t>
         </x:is>
       </x:c>
-      <x:c r="N8" s="63" t="inlineStr">
+      <x:c r="N8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">PV</x:t>
         </x:is>
@@ -2986,24 +2881,24 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="62" t="inlineStr">
+      <x:c r="A1" s="20" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">DCF - Bull scenario</x:t>
         </x:is>
       </x:c>
-      <x:c r="B1" s="62"/>
-      <x:c r="C1" s="62"/>
-      <x:c r="D1" s="62"/>
-      <x:c r="E1" s="62"/>
-      <x:c r="F1" s="62"/>
-      <x:c r="G1" s="62"/>
-      <x:c r="H1" s="62"/>
-      <x:c r="I1" s="62"/>
-      <x:c r="J1" s="62"/>
-      <x:c r="K1" s="62"/>
-      <x:c r="L1" s="62"/>
-      <x:c r="M1" s="62"/>
-      <x:c r="N1" s="62"/>
+      <x:c r="B1" s="20"/>
+      <x:c r="C1" s="20"/>
+      <x:c r="D1" s="20"/>
+      <x:c r="E1" s="20"/>
+      <x:c r="F1" s="20"/>
+      <x:c r="G1" s="20"/>
+      <x:c r="H1" s="20"/>
+      <x:c r="I1" s="20"/>
+      <x:c r="J1" s="20"/>
+      <x:c r="K1" s="20"/>
+      <x:c r="L1" s="20"/>
+      <x:c r="M1" s="20"/>
+      <x:c r="N1" s="20"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="17" t="inlineStr">
@@ -3132,72 +3027,72 @@
       <x:c r="N7" s="17"/>
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
-      <x:c r="A8" s="63" t="inlineStr">
+      <x:c r="A8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Year</x:t>
         </x:is>
       </x:c>
-      <x:c r="B8" s="63" t="inlineStr">
+      <x:c r="B8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">i</x:t>
         </x:is>
       </x:c>
-      <x:c r="C8" s="63" t="inlineStr">
+      <x:c r="C8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">growth</x:t>
         </x:is>
       </x:c>
-      <x:c r="D8" s="63" t="inlineStr">
+      <x:c r="D8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">revenue</x:t>
         </x:is>
       </x:c>
-      <x:c r="E8" s="63" t="inlineStr">
+      <x:c r="E8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">op margin</x:t>
         </x:is>
       </x:c>
-      <x:c r="F8" s="63" t="inlineStr">
+      <x:c r="F8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">EBIT</x:t>
         </x:is>
       </x:c>
-      <x:c r="G8" s="63" t="inlineStr">
+      <x:c r="G8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">cash tax</x:t>
         </x:is>
       </x:c>
-      <x:c r="H8" s="63" t="inlineStr">
+      <x:c r="H8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">NOL end</x:t>
         </x:is>
       </x:c>
-      <x:c r="I8" s="63" t="inlineStr">
+      <x:c r="I8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">NOPAT</x:t>
         </x:is>
       </x:c>
-      <x:c r="J8" s="63" t="inlineStr">
+      <x:c r="J8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">dRev</x:t>
         </x:is>
       </x:c>
-      <x:c r="K8" s="63" t="inlineStr">
+      <x:c r="K8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">reinvest</x:t>
         </x:is>
       </x:c>
-      <x:c r="L8" s="63" t="inlineStr">
+      <x:c r="L8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">FCFF</x:t>
         </x:is>
       </x:c>
-      <x:c r="M8" s="63" t="inlineStr">
+      <x:c r="M8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">disc</x:t>
         </x:is>
       </x:c>
-      <x:c r="N8" s="63" t="inlineStr">
+      <x:c r="N8" s="23" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">PV</x:t>
         </x:is>
@@ -3956,32 +3851,32 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="60" t="inlineStr">
+      <x:c r="A1" s="10" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">VALUATION SUMMARY</x:t>
         </x:is>
       </x:c>
-      <x:c r="B1" s="60"/>
-      <x:c r="C1" s="60"/>
-      <x:c r="D1" s="60"/>
+      <x:c r="B1" s="10"/>
+      <x:c r="C1" s="10"/>
+      <x:c r="D1" s="10"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="65" t="inlineStr">
+      <x:c r="A2" s="29" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Scenario</x:t>
         </x:is>
       </x:c>
-      <x:c r="B2" s="65" t="inlineStr">
+      <x:c r="B2" s="29" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Prob</x:t>
         </x:is>
       </x:c>
-      <x:c r="C2" s="65" t="inlineStr">
+      <x:c r="C2" s="29" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Equity (US$m)</x:t>
         </x:is>
       </x:c>
-      <x:c r="D2" s="65" t="inlineStr">
+      <x:c r="D2" s="29" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Per share (HK$)</x:t>
         </x:is>
@@ -4042,17 +3937,17 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="68" t="inlineStr">
+      <x:c r="A6" s="36" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">PROB-WEIGHTED</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" s="68"/>
-      <x:c r="C6" s="69" t="n">
+      <x:c r="B6" s="36"/>
+      <x:c r="C6" s="37" t="n">
         <x:f>SUMPRODUCT(B3:B5,C3:C5)/SUM(B3:B5)</x:f>
         <x:v>5252.4277585098625</x:v>
       </x:c>
-      <x:c r="D6" s="69" t="n">
+      <x:c r="D6" s="37" t="n">
         <x:f>SUMPRODUCT(B3:B5,D3:D5)/SUM(B3:B5)</x:f>
         <x:v>87.98733867853703</x:v>
       </x:c>
@@ -4086,12 +3981,12 @@
     <x:row r="9">
       <x:c r="A9" s="6" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Market equity value / revenue</x:t>
+          <x:t xml:space="preserve">Market equity value / LTM revenue</x:t>
         </x:is>
       </x:c>
       <x:c r="B9" s="31" t="n">
-        <x:f>(Assumptions!B9*Assumptions!B5/Assumptions!B6)/Assumptions!B11</x:f>
-        <x:v>101.90835028388278</x:v>
+        <x:f>(Assumptions!B9*Assumptions!B5/Assumptions!B6)/Assumptions!B12</x:f>
+        <x:v>340.5361345181736</x:v>
       </x:c>
       <x:c r="C9" s="6"/>
       <x:c r="D9" s="6"/>
@@ -4122,788 +4017,788 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="38" customHeight="1">
-      <x:c r="A1" s="70" t="inlineStr">
+      <x:c r="A1" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Company</x:t>
         </x:is>
       </x:c>
-      <x:c r="B1" s="70" t="inlineStr">
+      <x:c r="B1" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Ticker</x:t>
         </x:is>
       </x:c>
-      <x:c r="C1" s="70" t="inlineStr">
+      <x:c r="C1" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Cohort</x:t>
         </x:is>
       </x:c>
-      <x:c r="D1" s="70" t="inlineStr">
+      <x:c r="D1" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Valuation date</x:t>
         </x:is>
       </x:c>
-      <x:c r="E1" s="70" t="inlineStr">
+      <x:c r="E1" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Valuation basis</x:t>
         </x:is>
       </x:c>
-      <x:c r="F1" s="70" t="inlineStr">
+      <x:c r="F1" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Equity value (bn)</x:t>
         </x:is>
       </x:c>
-      <x:c r="G1" s="70" t="inlineStr">
+      <x:c r="G1" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Revenue (bn)</x:t>
         </x:is>
       </x:c>
-      <x:c r="H1" s="70" t="inlineStr">
+      <x:c r="H1" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Currency</x:t>
         </x:is>
       </x:c>
-      <x:c r="I1" s="70" t="inlineStr">
+      <x:c r="I1" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Revenue basis</x:t>
         </x:is>
       </x:c>
-      <x:c r="J1" s="70" t="inlineStr">
+      <x:c r="J1" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Private range flag</x:t>
         </x:is>
       </x:c>
-      <x:c r="K1" s="70" t="inlineStr">
+      <x:c r="K1" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Valuation source</x:t>
         </x:is>
       </x:c>
-      <x:c r="L1" s="70" t="inlineStr">
+      <x:c r="L1" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Revenue source</x:t>
         </x:is>
       </x:c>
-      <x:c r="M1" s="70" t="inlineStr">
+      <x:c r="M1" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Comparability note</x:t>
         </x:is>
       </x:c>
-      <x:c r="N1" s="70" t="inlineStr">
+      <x:c r="N1" s="41" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Equity value / revenue (x)</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
-      <x:c r="A2" s="71" t="inlineStr">
+      <x:c r="A2" s="44" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Zhipu</x:t>
         </x:is>
       </x:c>
-      <x:c r="B2" s="71" t="inlineStr">
+      <x:c r="B2" s="44" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">02513.HK</x:t>
         </x:is>
       </x:c>
-      <x:c r="C2" s="71" t="inlineStr">
+      <x:c r="C2" s="44" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">core_frontier</x:t>
         </x:is>
       </x:c>
-      <x:c r="D2" s="71" t="inlineStr">
+      <x:c r="D2" s="44" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-08-31</x:t>
         </x:is>
       </x:c>
-      <x:c r="E2" s="72" t="inlineStr">
+      <x:c r="E2" s="45" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">public market equity value</x:t>
         </x:is>
       </x:c>
-      <x:c r="F2" s="73" t="n">
+      <x:c r="F2" s="51" t="n">
         <x:v>71.33584519871795</x:v>
       </x:c>
-      <x:c r="G2" s="73" t="n">
-        <x:v>0.7</x:v>
-      </x:c>
-      <x:c r="H2" s="71" t="inlineStr">
+      <x:c r="G2" s="51" t="n">
+        <x:v>0.209480985915493</x:v>
+      </x:c>
+      <x:c r="H2" s="44" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">USD</x:t>
         </x:is>
       </x:c>
-      <x:c r="I2" s="72" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FY2026E model estimate anchored to H1 actual and August run-rate</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J2" s="71" t="n">
+      <x:c r="I2" s="45" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">LTM through 2026H1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J2" s="44" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K2" s="72" t="inlineStr">
+      <x:c r="K2" s="45" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www.hkex.com.hk/chi/stat/smstat/dayquot/d260831c.htm</x:t>
         </x:is>
       </x:c>
-      <x:c r="L2" s="72" t="inlineStr">
+      <x:c r="L2" s="45" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0831/2026083101539.pdf</x:t>
         </x:is>
       </x:c>
-      <x:c r="M2" s="72" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Subject company; equity value is refreshed from the local market file and post-placement share count; revenue is a model estimate rather than company guidance.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N2" s="74" t="n">
+      <x:c r="M2" s="45" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Subject company; equity value is refreshed from the local market file and post-placement share count; LTM revenue is FY2025 less H1 2025 plus H1 2026 and translated at USD/CNY 7.1.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N2" s="55" t="n">
         <x:f>F2/G2</x:f>
-        <x:v>101.90835028388278</x:v>
+        <x:v>340.5361345181736</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
-      <x:c r="A3" s="75" t="inlineStr">
+      <x:c r="A3" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">MiniMax</x:t>
         </x:is>
       </x:c>
-      <x:c r="B3" s="75" t="inlineStr">
+      <x:c r="B3" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">00100.HK</x:t>
         </x:is>
       </x:c>
-      <x:c r="C3" s="75" t="inlineStr">
+      <x:c r="C3" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">core_frontier</x:t>
         </x:is>
       </x:c>
-      <x:c r="D3" s="75" t="inlineStr">
+      <x:c r="D3" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-08-31</x:t>
         </x:is>
       </x:c>
-      <x:c r="E3" s="76" t="inlineStr">
+      <x:c r="E3" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">public market equity value</x:t>
         </x:is>
       </x:c>
-      <x:c r="F3" s="77" t="n">
+      <x:c r="F3" s="52" t="n">
         <x:v>15.626042</x:v>
       </x:c>
-      <x:c r="G3" s="77" t="n">
+      <x:c r="G3" s="52" t="n">
         <x:v>0.165182</x:v>
       </x:c>
-      <x:c r="H3" s="75" t="inlineStr">
+      <x:c r="H3" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">USD</x:t>
         </x:is>
       </x:c>
-      <x:c r="I3" s="76" t="inlineStr">
+      <x:c r="I3" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">LTM through 2026H1</x:t>
         </x:is>
       </x:c>
-      <x:c r="J3" s="75" t="n">
+      <x:c r="J3" s="46" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K3" s="76" t="inlineStr">
+      <x:c r="K3" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www.hkex.com.hk/chi/stat/smstat/dayquot/d260831c.htm</x:t>
         </x:is>
       </x:c>
-      <x:c r="L3" s="76" t="inlineStr">
+      <x:c r="L3" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0826/2026082600680.pdf</x:t>
         </x:is>
       </x:c>
-      <x:c r="M3" s="76" t="inlineStr">
+      <x:c r="M3" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Closest listed foundation-model peer; public-market LTM multiple is shown separately from private transaction references.</x:t>
         </x:is>
       </x:c>
-      <x:c r="N3" s="78" t="n">
+      <x:c r="N3" s="56" t="n">
         <x:f>F3/G3</x:f>
         <x:v>94.59893935174534</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
-      <x:c r="A4" s="75" t="inlineStr">
+      <x:c r="A4" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">OpenAI</x:t>
         </x:is>
       </x:c>
-      <x:c r="B4" s="75" t="inlineStr">
+      <x:c r="B4" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">private</x:t>
         </x:is>
       </x:c>
-      <x:c r="C4" s="75" t="inlineStr">
+      <x:c r="C4" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">core_frontier</x:t>
         </x:is>
       </x:c>
-      <x:c r="D4" s="75" t="inlineStr">
+      <x:c r="D4" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-03-31</x:t>
         </x:is>
       </x:c>
-      <x:c r="E4" s="76" t="inlineStr">
+      <x:c r="E4" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">post-money financing</x:t>
         </x:is>
       </x:c>
-      <x:c r="F4" s="77" t="n">
+      <x:c r="F4" s="52" t="n">
         <x:v>852</x:v>
       </x:c>
-      <x:c r="G4" s="77" t="n">
+      <x:c r="G4" s="52" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="H4" s="75" t="inlineStr">
+      <x:c r="H4" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">USD</x:t>
         </x:is>
       </x:c>
-      <x:c r="I4" s="76" t="inlineStr">
+      <x:c r="I4" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">annualized revenue at February 2026</x:t>
         </x:is>
       </x:c>
-      <x:c r="J4" s="75" t="n">
+      <x:c r="J4" s="46" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K4" s="76" t="inlineStr">
+      <x:c r="K4" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://openai.com/index/accelerating-the-next-phase-ai/</x:t>
         </x:is>
       </x:c>
-      <x:c r="L4" s="76" t="inlineStr">
+      <x:c r="L4" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://finance.yahoo.com/news/openai-tops-25-billion-annualized-033836274.html</x:t>
         </x:is>
       </x:c>
-      <x:c r="M4" s="76" t="inlineStr">
+      <x:c r="M4" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Private frontier-lab transaction reference; revenue was reported by Reuters and was not independently verified.</x:t>
         </x:is>
       </x:c>
-      <x:c r="N4" s="78" t="n">
+      <x:c r="N4" s="56" t="n">
         <x:f>F4/G4</x:f>
         <x:v>34.08</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
-      <x:c r="A5" s="75" t="inlineStr">
+      <x:c r="A5" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Anthropic</x:t>
         </x:is>
       </x:c>
-      <x:c r="B5" s="75" t="inlineStr">
+      <x:c r="B5" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">private</x:t>
         </x:is>
       </x:c>
-      <x:c r="C5" s="75" t="inlineStr">
+      <x:c r="C5" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">core_frontier</x:t>
         </x:is>
       </x:c>
-      <x:c r="D5" s="75" t="inlineStr">
+      <x:c r="D5" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-05-28</x:t>
         </x:is>
       </x:c>
-      <x:c r="E5" s="76" t="inlineStr">
+      <x:c r="E5" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">post-money financing</x:t>
         </x:is>
       </x:c>
-      <x:c r="F5" s="77" t="n">
+      <x:c r="F5" s="52" t="n">
         <x:v>965</x:v>
       </x:c>
-      <x:c r="G5" s="77" t="n">
+      <x:c r="G5" s="52" t="n">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="H5" s="75" t="inlineStr">
+      <x:c r="H5" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">USD</x:t>
         </x:is>
       </x:c>
-      <x:c r="I5" s="76" t="inlineStr">
+      <x:c r="I5" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">annualized revenue at May 2026</x:t>
         </x:is>
       </x:c>
-      <x:c r="J5" s="75" t="n">
+      <x:c r="J5" s="46" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K5" s="76" t="inlineStr">
+      <x:c r="K5" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www.anthropic.com/news/series-h</x:t>
         </x:is>
       </x:c>
-      <x:c r="L5" s="76" t="inlineStr">
+      <x:c r="L5" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www.anthropic.com/news/series-h</x:t>
         </x:is>
       </x:c>
-      <x:c r="M5" s="76" t="inlineStr">
+      <x:c r="M5" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Private frontier-lab transaction reference with valuation and revenue disclosed together by the company.</x:t>
         </x:is>
       </x:c>
-      <x:c r="N5" s="78" t="n">
+      <x:c r="N5" s="56" t="n">
         <x:f>F5/G5</x:f>
         <x:v>20.53191489361702</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
-      <x:c r="A6" s="75" t="inlineStr">
+      <x:c r="A6" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Mistral</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" s="75" t="inlineStr">
+      <x:c r="B6" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">private</x:t>
         </x:is>
       </x:c>
-      <x:c r="C6" s="75" t="inlineStr">
+      <x:c r="C6" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">core_frontier</x:t>
         </x:is>
       </x:c>
-      <x:c r="D6" s="75" t="inlineStr">
+      <x:c r="D6" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2025-09-09</x:t>
         </x:is>
       </x:c>
-      <x:c r="E6" s="76" t="inlineStr">
+      <x:c r="E6" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">post-money financing</x:t>
         </x:is>
       </x:c>
-      <x:c r="F6" s="77" t="n">
+      <x:c r="F6" s="52" t="n">
         <x:v>11.7</x:v>
       </x:c>
-      <x:c r="G6" s="77" t="n">
+      <x:c r="G6" s="52" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="H6" s="75" t="inlineStr">
+      <x:c r="H6" s="46" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">EUR</x:t>
         </x:is>
       </x:c>
-      <x:c r="I6" s="76" t="inlineStr">
+      <x:c r="I6" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">annualized revenue at September 2025</x:t>
         </x:is>
       </x:c>
-      <x:c r="J6" s="75" t="n">
+      <x:c r="J6" s="46" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K6" s="76" t="inlineStr">
+      <x:c r="K6" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://mistral.ai/news/mistral-ai-raises-1-7-b-to-accelerate-technological-progress-with-ai/</x:t>
         </x:is>
       </x:c>
-      <x:c r="L6" s="76" t="inlineStr">
+      <x:c r="L6" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www.lemonde.fr/economie/article/2025/09/26/mistral-ai-incarnation-de-l-intelligence-artificielle_6643087_3234.html</x:t>
         </x:is>
       </x:c>
-      <x:c r="M6" s="76" t="inlineStr">
+      <x:c r="M6" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Older private frontier-lab reference; included in the private transaction range but dated separately.</x:t>
         </x:is>
       </x:c>
-      <x:c r="N6" s="78" t="n">
+      <x:c r="N6" s="56" t="n">
         <x:f>F6/G6</x:f>
         <x:v>39</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
-      <x:c r="A7" s="79" t="inlineStr">
+      <x:c r="A7" s="48" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">SenseTime</x:t>
         </x:is>
       </x:c>
-      <x:c r="B7" s="79" t="inlineStr">
+      <x:c r="B7" s="48" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">00020.HK</x:t>
         </x:is>
       </x:c>
-      <x:c r="C7" s="79" t="inlineStr">
+      <x:c r="C7" s="48" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">hk_adjacent</x:t>
         </x:is>
       </x:c>
-      <x:c r="D7" s="79" t="inlineStr">
+      <x:c r="D7" s="48" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-08-31</x:t>
         </x:is>
       </x:c>
-      <x:c r="E7" s="80" t="inlineStr">
+      <x:c r="E7" s="49" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">implied total equity value</x:t>
         </x:is>
       </x:c>
-      <x:c r="F7" s="81" t="n">
+      <x:c r="F7" s="53" t="n">
         <x:v>52.58377</x:v>
       </x:c>
-      <x:c r="G7" s="81" t="n">
+      <x:c r="G7" s="53" t="n">
         <x:v>5.567388</x:v>
       </x:c>
-      <x:c r="H7" s="79" t="inlineStr">
+      <x:c r="H7" s="48" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">CNY</x:t>
         </x:is>
       </x:c>
-      <x:c r="I7" s="80" t="inlineStr">
+      <x:c r="I7" s="49" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">LTM through 2026H1</x:t>
         </x:is>
       </x:c>
-      <x:c r="J7" s="79" t="n">
+      <x:c r="J7" s="48" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K7" s="80" t="inlineStr">
+      <x:c r="K7" s="49" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www.hkex.com.hk/chi/stat/smstat/dayquot/d260831c.htm</x:t>
         </x:is>
       </x:c>
-      <x:c r="L7" s="80" t="inlineStr">
+      <x:c r="L7" s="49" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0826/2026082600408.pdf</x:t>
         </x:is>
       </x:c>
-      <x:c r="M7" s="80" t="inlineStr">
+      <x:c r="M7" s="49" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Adjacent Hong Kong AI platform; mixed computer-vision generative-AI and solution revenue makes it contextual only.</x:t>
         </x:is>
       </x:c>
-      <x:c r="N7" s="82" t="n">
+      <x:c r="N7" s="57" t="n">
         <x:f>F7/G7</x:f>
         <x:v>9.444962341406779</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
-      <x:c r="A8" s="79" t="inlineStr">
+      <x:c r="A8" s="48" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Phancy</x:t>
         </x:is>
       </x:c>
-      <x:c r="B8" s="79" t="inlineStr">
+      <x:c r="B8" s="48" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">06682.HK</x:t>
         </x:is>
       </x:c>
-      <x:c r="C8" s="79" t="inlineStr">
+      <x:c r="C8" s="48" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">hk_adjacent</x:t>
         </x:is>
       </x:c>
-      <x:c r="D8" s="79" t="inlineStr">
+      <x:c r="D8" s="48" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-08-31</x:t>
         </x:is>
       </x:c>
-      <x:c r="E8" s="80" t="inlineStr">
+      <x:c r="E8" s="49" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">implied total equity value</x:t>
         </x:is>
       </x:c>
-      <x:c r="F8" s="81" t="n">
+      <x:c r="F8" s="53" t="n">
         <x:v>13.500771</x:v>
       </x:c>
-      <x:c r="G8" s="81" t="n">
+      <x:c r="G8" s="53" t="n">
         <x:v>8.274082999999999</x:v>
       </x:c>
-      <x:c r="H8" s="79" t="inlineStr">
+      <x:c r="H8" s="48" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">CNY</x:t>
         </x:is>
       </x:c>
-      <x:c r="I8" s="80" t="inlineStr">
+      <x:c r="I8" s="49" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">LTM through 2026H1</x:t>
         </x:is>
       </x:c>
-      <x:c r="J8" s="79" t="n">
+      <x:c r="J8" s="48" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K8" s="80" t="inlineStr">
+      <x:c r="K8" s="49" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www.hkex.com.hk/chi/stat/smstat/dayquot/d260831c.htm</x:t>
         </x:is>
       </x:c>
-      <x:c r="L8" s="80" t="inlineStr">
+      <x:c r="L8" s="49" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0820/2026082000357.pdf</x:t>
         </x:is>
       </x:c>
-      <x:c r="M8" s="80" t="inlineStr">
+      <x:c r="M8" s="49" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Enterprise AI platform and agentic services with a different revenue and margin mix; contextual only.</x:t>
         </x:is>
       </x:c>
-      <x:c r="N8" s="82" t="n">
+      <x:c r="N8" s="57" t="n">
         <x:f>F8/G8</x:f>
         <x:v>1.6316939291036845</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
-      <x:c r="A9" s="79" t="inlineStr">
+      <x:c r="A9" s="48" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Wenge AI</x:t>
         </x:is>
       </x:c>
-      <x:c r="B9" s="79" t="inlineStr">
+      <x:c r="B9" s="48" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">01956.HK</x:t>
         </x:is>
       </x:c>
-      <x:c r="C9" s="79" t="inlineStr">
+      <x:c r="C9" s="48" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">hk_adjacent</x:t>
         </x:is>
       </x:c>
-      <x:c r="D9" s="79" t="inlineStr">
+      <x:c r="D9" s="48" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-08-31</x:t>
         </x:is>
       </x:c>
-      <x:c r="E9" s="80" t="inlineStr">
+      <x:c r="E9" s="49" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">implied total equity value</x:t>
         </x:is>
       </x:c>
-      <x:c r="F9" s="81" t="n">
+      <x:c r="F9" s="53" t="n">
         <x:v>12.976009</x:v>
       </x:c>
-      <x:c r="G9" s="81" t="n">
+      <x:c r="G9" s="53" t="n">
         <x:v>0.459773</x:v>
       </x:c>
-      <x:c r="H9" s="79" t="inlineStr">
+      <x:c r="H9" s="48" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">CNY</x:t>
         </x:is>
       </x:c>
-      <x:c r="I9" s="80" t="inlineStr">
+      <x:c r="I9" s="49" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">LTM through 2026H1</x:t>
         </x:is>
       </x:c>
-      <x:c r="J9" s="79" t="n">
+      <x:c r="J9" s="48" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K9" s="80" t="inlineStr">
+      <x:c r="K9" s="49" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www.hkex.com.hk/chi/stat/smstat/dayquot/d260831c.htm</x:t>
         </x:is>
       </x:c>
-      <x:c r="L9" s="80" t="inlineStr">
+      <x:c r="L9" s="49" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0825/2026082500959.pdf</x:t>
         </x:is>
       </x:c>
-      <x:c r="M9" s="80" t="inlineStr">
+      <x:c r="M9" s="49" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Decision-intelligence and project-delivery model with a short trading history; contextual only.</x:t>
         </x:is>
       </x:c>
-      <x:c r="N9" s="82" t="n">
+      <x:c r="N9" s="57" t="n">
         <x:f>F9/G9</x:f>
         <x:v>28.222642477918452</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
-      <x:c r="A10" s="83" t="inlineStr">
+      <x:c r="A10" s="32" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Palantir</x:t>
         </x:is>
       </x:c>
-      <x:c r="B10" s="83" t="inlineStr">
+      <x:c r="B10" s="32" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">PLTR</x:t>
         </x:is>
       </x:c>
-      <x:c r="C10" s="83" t="inlineStr">
+      <x:c r="C10" s="32" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">commercialization_reference</x:t>
         </x:is>
       </x:c>
-      <x:c r="D10" s="83" t="inlineStr">
+      <x:c r="D10" s="32" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-08-31</x:t>
         </x:is>
       </x:c>
-      <x:c r="E10" s="84" t="inlineStr">
+      <x:c r="E10" s="50" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">public market equity value</x:t>
         </x:is>
       </x:c>
-      <x:c r="F10" s="85" t="n">
+      <x:c r="F10" s="54" t="n">
         <x:v>447.856263</x:v>
       </x:c>
-      <x:c r="G10" s="85" t="n">
+      <x:c r="G10" s="54" t="n">
         <x:v>4.475446</x:v>
       </x:c>
-      <x:c r="H10" s="83" t="inlineStr">
+      <x:c r="H10" s="32" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">USD</x:t>
         </x:is>
       </x:c>
-      <x:c r="I10" s="84" t="inlineStr">
+      <x:c r="I10" s="50" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">FY2025 revenue</x:t>
         </x:is>
       </x:c>
-      <x:c r="J10" s="83" t="n">
+      <x:c r="J10" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K10" s="84" t="inlineStr">
+      <x:c r="K10" s="50" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www.gurufocus.com/stock/PLTR/data/market-cap</x:t>
         </x:is>
       </x:c>
-      <x:c r="L10" s="84" t="inlineStr">
+      <x:c r="L10" s="50" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www.sec.gov/Archives/edgar/data/1321655/000132165526000011/pltr-20251231.htm</x:t>
         </x:is>
       </x:c>
-      <x:c r="M10" s="84" t="inlineStr">
+      <x:c r="M10" s="50" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Mature AI software commercialization reference; not a frontier-model laboratory.</x:t>
         </x:is>
       </x:c>
-      <x:c r="N10" s="86" t="n">
+      <x:c r="N10" s="58" t="n">
         <x:f>F10/G10</x:f>
         <x:v>100.06963842262873</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
-      <x:c r="A11" s="83" t="inlineStr">
+      <x:c r="A11" s="32" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Cloudflare</x:t>
         </x:is>
       </x:c>
-      <x:c r="B11" s="83" t="inlineStr">
+      <x:c r="B11" s="32" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">NET</x:t>
         </x:is>
       </x:c>
-      <x:c r="C11" s="83" t="inlineStr">
+      <x:c r="C11" s="32" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">commercialization_reference</x:t>
         </x:is>
       </x:c>
-      <x:c r="D11" s="83" t="inlineStr">
+      <x:c r="D11" s="32" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-08-31</x:t>
         </x:is>
       </x:c>
-      <x:c r="E11" s="84" t="inlineStr">
+      <x:c r="E11" s="50" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">public market equity value</x:t>
         </x:is>
       </x:c>
-      <x:c r="F11" s="85" t="n">
+      <x:c r="F11" s="54" t="n">
         <x:v>108.259915</x:v>
       </x:c>
-      <x:c r="G11" s="85" t="n">
+      <x:c r="G11" s="54" t="n">
         <x:v>2.1679</x:v>
       </x:c>
-      <x:c r="H11" s="83" t="inlineStr">
+      <x:c r="H11" s="32" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">USD</x:t>
         </x:is>
       </x:c>
-      <x:c r="I11" s="84" t="inlineStr">
+      <x:c r="I11" s="50" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">FY2025 revenue</x:t>
         </x:is>
       </x:c>
-      <x:c r="J11" s="83" t="n">
+      <x:c r="J11" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K11" s="84" t="inlineStr">
+      <x:c r="K11" s="50" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www.tipranks.com/stocks/net/market-cap</x:t>
         </x:is>
       </x:c>
-      <x:c r="L11" s="84" t="inlineStr">
+      <x:c r="L11" s="50" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www.cloudflare.com/press/press-releases/2026/cloudflare-announces-fourth-quarter-and-fiscal-year-2025-financial-results/</x:t>
         </x:is>
       </x:c>
-      <x:c r="M11" s="84" t="inlineStr">
+      <x:c r="M11" s="50" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Connectivity and inference-infrastructure reference; economics differ from a model laboratory.</x:t>
         </x:is>
       </x:c>
-      <x:c r="N11" s="86" t="n">
+      <x:c r="N11" s="58" t="n">
         <x:f>F11/G11</x:f>
         <x:v>49.93768854651968</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
-      <x:c r="A12" s="83" t="inlineStr">
+      <x:c r="A12" s="32" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Snowflake</x:t>
         </x:is>
       </x:c>
-      <x:c r="B12" s="83" t="inlineStr">
+      <x:c r="B12" s="32" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">SNOW</x:t>
         </x:is>
       </x:c>
-      <x:c r="C12" s="83" t="inlineStr">
+      <x:c r="C12" s="32" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">commercialization_reference</x:t>
         </x:is>
       </x:c>
-      <x:c r="D12" s="83" t="inlineStr">
+      <x:c r="D12" s="32" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-08-31</x:t>
         </x:is>
       </x:c>
-      <x:c r="E12" s="84" t="inlineStr">
+      <x:c r="E12" s="50" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">public market equity value</x:t>
         </x:is>
       </x:c>
-      <x:c r="F12" s="85" t="n">
+      <x:c r="F12" s="54" t="n">
         <x:v>114.87384</x:v>
       </x:c>
-      <x:c r="G12" s="85" t="n">
+      <x:c r="G12" s="54" t="n">
         <x:v>4.683946</x:v>
       </x:c>
-      <x:c r="H12" s="83" t="inlineStr">
+      <x:c r="H12" s="32" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">USD</x:t>
         </x:is>
       </x:c>
-      <x:c r="I12" s="84" t="inlineStr">
+      <x:c r="I12" s="50" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">FY2026 revenue</x:t>
         </x:is>
       </x:c>
-      <x:c r="J12" s="83" t="n">
+      <x:c r="J12" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K12" s="84" t="inlineStr">
+      <x:c r="K12" s="50" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://finance.yahoo.com/quote/SNOW/history/</x:t>
         </x:is>
       </x:c>
-      <x:c r="L12" s="84" t="inlineStr">
+      <x:c r="L12" s="50" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www.sec.gov/Archives/edgar/data/1640147/000164014726000023/snowflake2026ars.pdf</x:t>
         </x:is>
       </x:c>
-      <x:c r="M12" s="84" t="inlineStr">
+      <x:c r="M12" s="50" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Data-cloud commercialization reference; not a direct foundation-model comparable.</x:t>
         </x:is>
       </x:c>
-      <x:c r="N12" s="86" t="n">
+      <x:c r="N12" s="58" t="n">
         <x:f>F12/G12</x:f>
         <x:v>24.525013738416284</x:v>
       </x:c>
@@ -4922,12 +4817,12 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="88" t="inlineStr">
+      <x:c r="A1" s="28" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Market date</x:t>
         </x:is>
       </x:c>
-      <x:c r="B1" s="88" t="inlineStr">
+      <x:c r="B1" s="28" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">2026-08-31</x:t>
         </x:is>
@@ -4956,11 +4851,11 @@
     <x:row r="4">
       <x:c r="A4" s="6" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Market equity value / FY2026E revenue</x:t>
+          <x:t xml:space="preserve">Market equity value / LTM revenue</x:t>
         </x:is>
       </x:c>
       <x:c r="B4" s="14" t="n">
-        <x:v>101.9</x:v>
+        <x:v>340.5</x:v>
       </x:c>
     </x:row>
     <x:row r="5">

</xml_diff>

<commit_message>
Update Zhipu valuation and market data through 2026-09-11
</commit_message>
<xml_diff>
--- a/model/valuation_model.xlsx
+++ b/model/valuation_model.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="Rc240d3ab765242df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bear" sheetId="2" r:id="R09f01bfdb4954575"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="3" r:id="R42ed4a9da89b4c29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull" sheetId="4" r:id="Rc3b6c825c8f0487d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="Rff5c854a24284c05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Comps" sheetId="6" r:id="Red3020c606e74f88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="7" r:id="R2372e65b90254933"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="Re0521b6859294264"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bear" sheetId="2" r:id="R44d84f7bfd3d4198"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="3" r:id="R3abba42f21bf42ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull" sheetId="4" r:id="R352b5aa4fadc400b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="R548ac8ef86e348b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Comps" sheetId="6" r:id="R96c2ebb06e1d499e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="7" r:id="R7ffadd3e9a7e46bc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -697,10 +697,8 @@
           <x:t xml:space="preserve">Market date</x:t>
         </x:is>
       </x:c>
-      <x:c r="B8" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-31</x:t>
-        </x:is>
+      <x:c r="B8" s="14" t="str">
+        <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="C8" s="11" t="inlineStr">
         <x:is>
@@ -715,7 +713,7 @@
         </x:is>
       </x:c>
       <x:c r="B9" s="14" t="n">
-        <x:v>1195</x:v>
+        <x:v>793</x:v>
       </x:c>
       <x:c r="C9" s="11"/>
     </x:row>
@@ -3960,7 +3958,7 @@
       </x:c>
       <x:c r="B7" s="14" t="n">
         <x:f>Assumptions!B9</x:f>
-        <x:v>1195</x:v>
+        <x:v>793</x:v>
       </x:c>
       <x:c r="C7" s="6"/>
       <x:c r="D7" s="6"/>
@@ -3973,7 +3971,7 @@
       </x:c>
       <x:c r="B8" s="12" t="n">
         <x:f>D6/B7</x:f>
-        <x:v>0.07362957211593056</x:v>
+        <x:v>0.1109550298594414</x:v>
       </x:c>
       <x:c r="C8" s="6"/>
       <x:c r="D8" s="6"/>
@@ -3986,7 +3984,7 @@
       </x:c>
       <x:c r="B9" s="31" t="n">
         <x:f>(Assumptions!B9*Assumptions!B5/Assumptions!B6)/Assumptions!B12</x:f>
-        <x:v>340.5361345181736</x:v>
+        <x:v>225.97920893130686</x:v>
       </x:c>
       <x:c r="C9" s="6"/>
       <x:c r="D9" s="6"/>
@@ -4104,10 +4102,8 @@
           <x:t xml:space="preserve">core_frontier</x:t>
         </x:is>
       </x:c>
-      <x:c r="D2" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-31</x:t>
-        </x:is>
+      <x:c r="D2" s="44" t="str">
+        <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="E2" s="45" t="inlineStr">
         <x:is>
@@ -4115,7 +4111,7 @@
         </x:is>
       </x:c>
       <x:c r="F2" s="51" t="n">
-        <x:v>71.33584519871795</x:v>
+        <x:v>47.33834748333334</x:v>
       </x:c>
       <x:c r="G2" s="51" t="n">
         <x:v>0.209480985915493</x:v>
@@ -4133,24 +4129,20 @@
       <x:c r="J2" s="44" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K2" s="45" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.hkex.com.hk/chi/stat/smstat/dayquot/d260831c.htm</x:t>
-        </x:is>
+      <x:c r="K2" s="45" t="str">
+        <x:v>https://web.ifzq.gtimg.cn/appstock/app/hkfqkline/get</x:v>
       </x:c>
       <x:c r="L2" s="45" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0831/2026083101539.pdf</x:t>
         </x:is>
       </x:c>
-      <x:c r="M2" s="45" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Subject company; equity value is refreshed from the local market file and post-placement share count; LTM revenue is FY2025 less H1 2025 plus H1 2026 and translated at USD/CNY 7.1.</x:t>
-        </x:is>
+      <x:c r="M2" s="45" t="str">
+        <x:v>Subject company; equity value is refreshed from the local market file and post-placement share count; LTM revenue is FY2025 less H1 2025 plus H1 2026 and translated at USD/CNY 7.1.</x:v>
       </x:c>
       <x:c r="N2" s="55" t="n">
         <x:f>F2/G2</x:f>
-        <x:v>340.5361345181736</x:v>
+        <x:v>225.97920893130683</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
@@ -4169,10 +4161,8 @@
           <x:t xml:space="preserve">core_frontier</x:t>
         </x:is>
       </x:c>
-      <x:c r="D3" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-31</x:t>
-        </x:is>
+      <x:c r="D3" s="46" t="str">
+        <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="E3" s="47" t="inlineStr">
         <x:is>
@@ -4180,7 +4170,7 @@
         </x:is>
       </x:c>
       <x:c r="F3" s="52" t="n">
-        <x:v>15.626042</x:v>
+        <x:v>12.088915014326648</x:v>
       </x:c>
       <x:c r="G3" s="52" t="n">
         <x:v>0.165182</x:v>
@@ -4198,24 +4188,20 @@
       <x:c r="J3" s="46" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K3" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.hkex.com.hk/chi/stat/smstat/dayquot/d260831c.htm</x:t>
-        </x:is>
+      <x:c r="K3" s="47" t="str">
+        <x:v>https://web.ifzq.gtimg.cn/appstock/app/hkfqkline/get</x:v>
       </x:c>
       <x:c r="L3" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0826/2026082600680.pdf</x:t>
         </x:is>
       </x:c>
-      <x:c r="M3" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Closest listed foundation-model peer; public-market LTM multiple is shown separately from private transaction references.</x:t>
-        </x:is>
+      <x:c r="M3" s="47" t="str">
+        <x:v>Closest listed foundation-model peer; public-market LTM multiple is shown separately from private transaction references. Price refreshed to 2026-09-11; share-count and FX basis carried forward from the 2026-08-31 snapshot.</x:v>
       </x:c>
       <x:c r="N3" s="56" t="n">
         <x:f>F3/G3</x:f>
-        <x:v>94.59893935174534</x:v>
+        <x:v>73.18542585951647</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
@@ -4559,10 +4545,8 @@
           <x:t xml:space="preserve">hk_adjacent</x:t>
         </x:is>
       </x:c>
-      <x:c r="D9" s="48" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-31</x:t>
-        </x:is>
+      <x:c r="D9" s="48" t="str">
+        <x:v>2026-09-11</x:v>
       </x:c>
       <x:c r="E9" s="49" t="inlineStr">
         <x:is>
@@ -4570,7 +4554,7 @@
         </x:is>
       </x:c>
       <x:c r="F9" s="53" t="n">
-        <x:v>12.976009</x:v>
+        <x:v>11.96508736860465</x:v>
       </x:c>
       <x:c r="G9" s="53" t="n">
         <x:v>0.459773</x:v>
@@ -4588,24 +4572,20 @@
       <x:c r="J9" s="48" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K9" s="49" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.hkex.com.hk/chi/stat/smstat/dayquot/d260831c.htm</x:t>
-        </x:is>
+      <x:c r="K9" s="49" t="str">
+        <x:v>https://web.ifzq.gtimg.cn/appstock/app/hkfqkline/get</x:v>
       </x:c>
       <x:c r="L9" s="49" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0825/2026082500959.pdf</x:t>
         </x:is>
       </x:c>
-      <x:c r="M9" s="49" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Decision-intelligence and project-delivery model with a short trading history; contextual only.</x:t>
-        </x:is>
+      <x:c r="M9" s="49" t="str">
+        <x:v>Decision-intelligence and project-delivery model with a short trading history; contextual only. Price refreshed to 2026-09-11; share-count and FX basis carried forward from the 2026-08-31 snapshot.</x:v>
       </x:c>
       <x:c r="N9" s="57" t="n">
         <x:f>F9/G9</x:f>
-        <x:v>28.222642477918452</x:v>
+        <x:v>26.02390172673178</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -4817,105 +4797,83 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Market date</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-31</x:t>
-        </x:is>
+      <x:c r="A1" s="28" t="str">
+        <x:v>Market date</x:v>
+      </x:c>
+      <x:c r="B1" s="28" t="str">
+        <x:v>2026-09-11</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Market price (HK$)</x:t>
-        </x:is>
+      <x:c r="A2" s="6" t="str">
+        <x:v>Market price (HK$)</x:v>
       </x:c>
       <x:c r="B2" s="14" t="n">
-        <x:v>1195</x:v>
+        <x:v>793</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Market equity value (US$m)</x:t>
-        </x:is>
+      <x:c r="A3" s="6" t="str">
+        <x:v>Market equity value (US$m)</x:v>
       </x:c>
       <x:c r="B3" s="14" t="n">
-        <x:v>71335.8</x:v>
+        <x:v>47338.3</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Market equity value / LTM revenue</x:t>
-        </x:is>
+      <x:c r="A4" s="6" t="str">
+        <x:v>Market equity value / LTM revenue</x:v>
       </x:c>
       <x:c r="B4" s="14" t="n">
-        <x:v>340.5</x:v>
+        <x:v>226</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Bear per share (HK$)</x:t>
-        </x:is>
+      <x:c r="A5" s="6" t="str">
+        <x:v>Bear per share (HK$)</x:v>
       </x:c>
       <x:c r="B5" s="14" t="n">
         <x:v>24.6</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Base per share (HK$)</x:t>
-        </x:is>
+      <x:c r="A6" s="6" t="str">
+        <x:v>Base per share (HK$)</x:v>
       </x:c>
       <x:c r="B6" s="14" t="n">
         <x:v>72.8</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Bull per share (HK$)</x:t>
-        </x:is>
+      <x:c r="A7" s="6" t="str">
+        <x:v>Bull per share (HK$)</x:v>
       </x:c>
       <x:c r="B7" s="14" t="n">
         <x:v>233.1</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Probability-weighted equity (US$m)</x:t>
-        </x:is>
+      <x:c r="A8" s="6" t="str">
+        <x:v>Probability-weighted equity (US$m)</x:v>
       </x:c>
       <x:c r="B8" s="14" t="n">
         <x:v>5252.4</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Probability-weighted per share (HK$)</x:t>
-        </x:is>
+      <x:c r="A9" s="6" t="str">
+        <x:v>Probability-weighted per share (HK$)</x:v>
       </x:c>
       <x:c r="B9" s="14" t="n">
         <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DCF value as % of market</x:t>
-        </x:is>
+      <x:c r="A10" s="6" t="str">
+        <x:v>DCF value as % of market</x:v>
       </x:c>
       <x:c r="B10" s="12" t="n">
-        <x:v>0.0736</x:v>
+        <x:v>0.111</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Update September 18 data and integrate product trust events
</commit_message>
<xml_diff>
--- a/model/valuation_model.xlsx
+++ b/model/valuation_model.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="Re0521b6859294264"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bear" sheetId="2" r:id="R44d84f7bfd3d4198"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="3" r:id="R3abba42f21bf42ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull" sheetId="4" r:id="R352b5aa4fadc400b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="R548ac8ef86e348b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Comps" sheetId="6" r:id="R96c2ebb06e1d499e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="7" r:id="R7ffadd3e9a7e46bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="R1a44555c839e4da9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bear" sheetId="2" r:id="R0a02c5940c404366"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="3" r:id="R664eec7b412f4578"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull" sheetId="4" r:id="R936addd43d9145dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="R0de6b5c3e9f044e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Comps" sheetId="6" r:id="Re7e2be1957eb48a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="7" r:id="Ra39dad12fd064ada"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -154,7 +154,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="59">
+  <x:cellXfs count="60">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -316,6 +316,7 @@
     <x:xf numFmtId="204" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -661,7 +662,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="13" t="n">
-        <x:v>465.62309</x:v>
+        <x:v>487.58809</x:v>
       </x:c>
       <x:c r="C5" s="11"/>
     </x:row>
@@ -683,12 +684,10 @@
         </x:is>
       </x:c>
       <x:c r="B7" s="14" t="n">
-        <x:v>4289.424135066811</x:v>
-      </x:c>
-      <x:c r="C7" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-06-30 cash + short-term FVPL investments less bank loans and leases, plus July placement net proceeds; not a reported 2026-08-31 cash balance</x:t>
-        </x:is>
+        <x:v>6307.779114018209</x:v>
+      </x:c>
+      <x:c r="C7" s="11" t="str">
+        <x:v>June net cash plus July and September placements; CB net proceeds less issue-date principal proxy. Excludes undisclosed cash burn.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -698,7 +697,7 @@
         </x:is>
       </x:c>
       <x:c r="B8" s="14" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-18</x:v>
       </x:c>
       <x:c r="C8" s="11" t="inlineStr">
         <x:is>
@@ -713,7 +712,7 @@
         </x:is>
       </x:c>
       <x:c r="B9" s="14" t="n">
-        <x:v>793</x:v>
+        <x:v>780</x:v>
       </x:c>
       <x:c r="C9" s="11"/>
     </x:row>
@@ -891,6 +890,50 @@
         <x:is>
           <x:t xml:space="preserve">interim results announcement did not include a cash-flow statement</x:t>
         </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>September placement net (HKD m)</x:v>
+      </x:c>
+      <x:c r="B24" s="59" t="n">
+        <x:v>15664.13</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>Completed 2026-09-16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>September CB net (USD m)</x:v>
+      </x:c>
+      <x:c r="B25" s="59" t="n">
+        <x:v>3010.77</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>Issued 2026-09-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>CB principal proxy (USD m)</x:v>
+      </x:c>
+      <x:c r="B26" s="59" t="n">
+        <x:v>3000.636815920398</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>3015.64 / 1.005; issue-date proxy, not IFRS fair value</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>September financing source</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>https://www.hkexnews.hk/listedco/listconews/sehk/2026/0918/2026091800400_c.pdf</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>Settlement / FX terms in September 13 announcement</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1812,7 +1855,7 @@
       </x:c>
       <x:c r="B24" s="25" t="n">
         <x:f>B23+Assumptions!$B$7</x:f>
-        <x:v>1470.5938252172482</x:v>
+        <x:v>3488.9488041686463</x:v>
       </x:c>
       <x:c r="C24" s="17"/>
       <x:c r="D24" s="17"/>
@@ -1835,7 +1878,7 @@
       </x:c>
       <x:c r="B25" s="25" t="n">
         <x:f>B24/Assumptions!$B$5</x:f>
-        <x:v>3.1583352647250553</x:v>
+        <x:v>7.155525074799605</x:v>
       </x:c>
       <x:c r="C25" s="17"/>
       <x:c r="D25" s="17"/>
@@ -1858,7 +1901,7 @@
       </x:c>
       <x:c r="B26" s="25" t="n">
         <x:f>B25*Assumptions!$B$6</x:f>
-        <x:v>24.63501506485543</x:v>
+        <x:v>55.81309558343691</x:v>
       </x:c>
       <x:c r="C26" s="17"/>
       <x:c r="D26" s="17"/>
@@ -2792,7 +2835,7 @@
       </x:c>
       <x:c r="B24" s="25" t="n">
         <x:f>B23+Assumptions!$B$7</x:f>
-        <x:v>4344.218166227473</x:v>
+        <x:v>6362.5731451788715</x:v>
       </x:c>
       <x:c r="C24" s="17"/>
       <x:c r="D24" s="17"/>
@@ -2815,7 +2858,7 @@
       </x:c>
       <x:c r="B25" s="25" t="n">
         <x:f>B24/Assumptions!$B$5</x:f>
-        <x:v>9.329902789458902</x:v>
+        <x:v>13.049074158433344</x:v>
       </x:c>
       <x:c r="C25" s="17"/>
       <x:c r="D25" s="17"/>
@@ -2838,7 +2881,7 @@
       </x:c>
       <x:c r="B26" s="25" t="n">
         <x:f>B25*Assumptions!$B$6</x:f>
-        <x:v>72.77324175777943</x:v>
+        <x:v>101.78277843578007</x:v>
       </x:c>
       <x:c r="C26" s="17"/>
       <x:c r="D26" s="17"/>
@@ -3772,7 +3815,7 @@
       </x:c>
       <x:c r="B24" s="25" t="n">
         <x:f>B23+Assumptions!$B$7</x:f>
-        <x:v>13914.108724407311</x:v>
+        <x:v>15932.46370335871</x:v>
       </x:c>
       <x:c r="C24" s="17"/>
       <x:c r="D24" s="17"/>
@@ -3795,7 +3838,7 @@
       </x:c>
       <x:c r="B25" s="25" t="n">
         <x:f>B24/Assumptions!$B$5</x:f>
-        <x:v>29.882772188997997</x:v>
+        <x:v>32.67607234491455</x:v>
       </x:c>
       <x:c r="C25" s="17"/>
       <x:c r="D25" s="17"/>
@@ -3818,7 +3861,7 @@
       </x:c>
       <x:c r="B26" s="25" t="n">
         <x:f>B25*Assumptions!$B$6</x:f>
-        <x:v>233.08562307418438</x:v>
+        <x:v>254.87336429033348</x:v>
       </x:c>
       <x:c r="C26" s="17"/>
       <x:c r="D26" s="17"/>
@@ -3891,11 +3934,11 @@
       </x:c>
       <x:c r="C3" s="14" t="n">
         <x:f>Bear!B24</x:f>
-        <x:v>1470.5938252172482</x:v>
+        <x:v>3488.9488041686463</x:v>
       </x:c>
       <x:c r="D3" s="14" t="n">
         <x:f>Bear!B26</x:f>
-        <x:v>24.63501506485543</x:v>
+        <x:v>55.81309558343691</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -3909,11 +3952,11 @@
       </x:c>
       <x:c r="C4" s="14" t="n">
         <x:f>Base!B24</x:f>
-        <x:v>4344.218166227473</x:v>
+        <x:v>6362.5731451788715</x:v>
       </x:c>
       <x:c r="D4" s="14" t="n">
         <x:f>Base!B26</x:f>
-        <x:v>72.77324175777943</x:v>
+        <x:v>101.78277843578007</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -3927,11 +3970,11 @@
       </x:c>
       <x:c r="C5" s="14" t="n">
         <x:f>Bull!B24</x:f>
-        <x:v>13914.108724407311</x:v>
+        <x:v>15932.46370335871</x:v>
       </x:c>
       <x:c r="D5" s="14" t="n">
         <x:f>Bull!B26</x:f>
-        <x:v>233.08562307418438</x:v>
+        <x:v>254.87336429033348</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -3943,11 +3986,11 @@
       <x:c r="B6" s="36"/>
       <x:c r="C6" s="37" t="n">
         <x:f>SUMPRODUCT(B3:B5,C3:C5)/SUM(B3:B5)</x:f>
-        <x:v>5252.4277585098625</x:v>
+        <x:v>7270.782737461261</x:v>
       </x:c>
       <x:c r="D6" s="37" t="n">
         <x:f>SUMPRODUCT(B3:B5,D3:D5)/SUM(B3:B5)</x:f>
-        <x:v>87.98733867853703</x:v>
+        <x:v>116.31150660837065</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -3958,7 +4001,7 @@
       </x:c>
       <x:c r="B7" s="14" t="n">
         <x:f>Assumptions!B9</x:f>
-        <x:v>793</x:v>
+        <x:v>780</x:v>
       </x:c>
       <x:c r="C7" s="6"/>
       <x:c r="D7" s="6"/>
@@ -3971,7 +4014,7 @@
       </x:c>
       <x:c r="B8" s="12" t="n">
         <x:f>D6/B7</x:f>
-        <x:v>0.1109550298594414</x:v>
+        <x:v>0.14911731616457777</x:v>
       </x:c>
       <x:c r="C8" s="6"/>
       <x:c r="D8" s="6"/>
@@ -3984,7 +4027,7 @@
       </x:c>
       <x:c r="B9" s="31" t="n">
         <x:f>(Assumptions!B9*Assumptions!B5/Assumptions!B6)/Assumptions!B12</x:f>
-        <x:v>225.97920893130686</x:v>
+        <x:v>232.76007026083917</x:v>
       </x:c>
       <x:c r="C9" s="6"/>
       <x:c r="D9" s="6"/>
@@ -4103,7 +4146,7 @@
         </x:is>
       </x:c>
       <x:c r="D2" s="44" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-18</x:v>
       </x:c>
       <x:c r="E2" s="45" t="inlineStr">
         <x:is>
@@ -4111,7 +4154,7 @@
         </x:is>
       </x:c>
       <x:c r="F2" s="51" t="n">
-        <x:v>47.33834748333334</x:v>
+        <x:v>48.75880900000001</x:v>
       </x:c>
       <x:c r="G2" s="51" t="n">
         <x:v>0.209480985915493</x:v>
@@ -4142,7 +4185,7 @@
       </x:c>
       <x:c r="N2" s="55" t="n">
         <x:f>F2/G2</x:f>
-        <x:v>225.97920893130683</x:v>
+        <x:v>232.76007026083914</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
@@ -4162,7 +4205,7 @@
         </x:is>
       </x:c>
       <x:c r="D3" s="46" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-18</x:v>
       </x:c>
       <x:c r="E3" s="47" t="inlineStr">
         <x:is>
@@ -4170,7 +4213,7 @@
         </x:is>
       </x:c>
       <x:c r="F3" s="52" t="n">
-        <x:v>12.088915014326648</x:v>
+        <x:v>13.566449071633238</x:v>
       </x:c>
       <x:c r="G3" s="52" t="n">
         <x:v>0.165182</x:v>
@@ -4197,11 +4240,11 @@
         </x:is>
       </x:c>
       <x:c r="M3" s="47" t="str">
-        <x:v>Closest listed foundation-model peer; public-market LTM multiple is shown separately from private transaction references. Price refreshed to 2026-09-11; share-count and FX basis carried forward from the 2026-08-31 snapshot.</x:v>
+        <x:v>Closest listed foundation-model peer; public-market LTM multiple is shown separately from private transaction references. Price refreshed to 2026-09-11; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-17; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-18; share-count and FX basis carried forward from the 2026-08-31 snapshot.</x:v>
       </x:c>
       <x:c r="N3" s="56" t="n">
         <x:f>F3/G3</x:f>
-        <x:v>73.18542585951647</x:v>
+        <x:v>82.13031124234625</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
@@ -4546,7 +4589,7 @@
         </x:is>
       </x:c>
       <x:c r="D9" s="48" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-18</x:v>
       </x:c>
       <x:c r="E9" s="49" t="inlineStr">
         <x:is>
@@ -4554,7 +4597,7 @@
         </x:is>
       </x:c>
       <x:c r="F9" s="53" t="n">
-        <x:v>11.96508736860465</x:v>
+        <x:v>12.025440898837209</x:v>
       </x:c>
       <x:c r="G9" s="53" t="n">
         <x:v>0.459773</x:v>
@@ -4581,11 +4624,11 @@
         </x:is>
       </x:c>
       <x:c r="M9" s="49" t="str">
-        <x:v>Decision-intelligence and project-delivery model with a short trading history; contextual only. Price refreshed to 2026-09-11; share-count and FX basis carried forward from the 2026-08-31 snapshot.</x:v>
+        <x:v>Decision-intelligence and project-delivery model with a short trading history; contextual only. Price refreshed to 2026-09-11; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-18; share-count and FX basis carried forward from the 2026-08-31 snapshot.</x:v>
       </x:c>
       <x:c r="N9" s="57" t="n">
         <x:f>F9/G9</x:f>
-        <x:v>26.02390172673178</x:v>
+        <x:v>26.15516983128024</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -4801,7 +4844,7 @@
         <x:v>Market date</x:v>
       </x:c>
       <x:c r="B1" s="28" t="str">
-        <x:v>2026-09-11</x:v>
+        <x:v>2026-09-18</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -4809,7 +4852,7 @@
         <x:v>Market price (HK$)</x:v>
       </x:c>
       <x:c r="B2" s="14" t="n">
-        <x:v>793</x:v>
+        <x:v>780</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4817,7 +4860,7 @@
         <x:v>Market equity value (US$m)</x:v>
       </x:c>
       <x:c r="B3" s="14" t="n">
-        <x:v>47338.3</x:v>
+        <x:v>48758.8</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -4825,7 +4868,7 @@
         <x:v>Market equity value / LTM revenue</x:v>
       </x:c>
       <x:c r="B4" s="14" t="n">
-        <x:v>226</x:v>
+        <x:v>232.8</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -4833,7 +4876,7 @@
         <x:v>Bear per share (HK$)</x:v>
       </x:c>
       <x:c r="B5" s="14" t="n">
-        <x:v>24.6</x:v>
+        <x:v>55.8</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -4841,7 +4884,7 @@
         <x:v>Base per share (HK$)</x:v>
       </x:c>
       <x:c r="B6" s="14" t="n">
-        <x:v>72.8</x:v>
+        <x:v>101.8</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -4849,7 +4892,7 @@
         <x:v>Bull per share (HK$)</x:v>
       </x:c>
       <x:c r="B7" s="14" t="n">
-        <x:v>233.1</x:v>
+        <x:v>254.9</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -4857,7 +4900,7 @@
         <x:v>Probability-weighted equity (US$m)</x:v>
       </x:c>
       <x:c r="B8" s="14" t="n">
-        <x:v>5252.4</x:v>
+        <x:v>7270.8</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4865,7 +4908,7 @@
         <x:v>Probability-weighted per share (HK$)</x:v>
       </x:c>
       <x:c r="B9" s="14" t="n">
-        <x:v>88</x:v>
+        <x:v>116.3</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -4873,7 +4916,7 @@
         <x:v>DCF value as % of market</x:v>
       </x:c>
       <x:c r="B10" s="12" t="n">
-        <x:v>0.111</x:v>
+        <x:v>0.1491</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Update September 30 valuation and add Anthropic IPO comparison
</commit_message>
<xml_diff>
--- a/model/valuation_model.xlsx
+++ b/model/valuation_model.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="R1a44555c839e4da9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bear" sheetId="2" r:id="R0a02c5940c404366"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="3" r:id="R664eec7b412f4578"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull" sheetId="4" r:id="R936addd43d9145dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="R0de6b5c3e9f044e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Comps" sheetId="6" r:id="Re7e2be1957eb48a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="7" r:id="Ra39dad12fd064ada"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="Ra8b8c6446c454431"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bear" sheetId="2" r:id="R9d9269088fc449f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="3" r:id="R13f6ad149da64d7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull" sheetId="4" r:id="Refd2ecf0c1354b8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="R84d50c8ccc0a40c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Comps" sheetId="6" r:id="Refda385eb32745b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="7" r:id="R81ac4e99dcdd4e31"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,13 +19,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="200" formatCode="0.0%"/>
     <x:numFmt numFmtId="201" formatCode="0.000"/>
     <x:numFmt numFmtId="202" formatCode="#,##0.0"/>
     <x:numFmt numFmtId="203" formatCode="0%"/>
     <x:numFmt numFmtId="204" formatCode="0.0&quot;x&quot;"/>
     <x:numFmt numFmtId="205" formatCode="#,##0.000"/>
+    <x:numFmt numFmtId="206" formatCode="#,##0.0;(#,##0.0);&quot;-&quot;"/>
   </x:numFmts>
   <x:fonts count="7">
     <x:font>
@@ -154,7 +155,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="60">
+  <x:cellXfs count="62">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -317,6 +318,10 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -684,10 +689,11 @@
         </x:is>
       </x:c>
       <x:c r="B7" s="14" t="n">
-        <x:v>6307.779114018209</x:v>
+        <x:f>(B20-B28-B21)/B29+(B22+B24)/B6+B25-B26</x:f>
+        <x:v>6292.850240778773</x:v>
       </x:c>
       <x:c r="C7" s="11" t="str">
-        <x:v>June net cash plus July and September placements; CB net proceeds less issue-date principal proxy. Excludes undisclosed cash burn.</x:v>
+        <x:v>June net cash excludes restricted deposits; adds July/September funding less CB principal proxy. Excludes subsequent cash burn.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -697,7 +703,7 @@
         </x:is>
       </x:c>
       <x:c r="B8" s="14" t="str">
-        <x:v>2026-09-18</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="C8" s="11" t="inlineStr">
         <x:is>
@@ -712,7 +718,7 @@
         </x:is>
       </x:c>
       <x:c r="B9" s="14" t="n">
-        <x:v>780</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="C9" s="11"/>
     </x:row>
@@ -876,20 +882,14 @@
       <x:c r="C22" s="11"/>
     </x:row>
     <x:row r="23" ht="36" customHeight="1">
-      <x:c r="A23" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026H1 operating cash flow</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B23" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not disclosed</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C23" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">interim results announcement did not include a cash-flow statement</x:t>
-        </x:is>
+      <x:c r="A23" s="6" t="str">
+        <x:v>2026H1 operating cash flow (RMB m)</x:v>
+      </x:c>
+      <x:c r="B23" s="60" t="n">
+        <x:v>-3374.057</x:v>
+      </x:c>
+      <x:c r="C23" s="11" t="str">
+        <x:v>Interim report pp.60-61; published 2026-09-24</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -934,6 +934,28 @@
       </x:c>
       <x:c r="C27" t="str">
         <x:v>Settlement / FX terms in September 13 announcement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>June restricted cash (RMB m)</x:v>
+      </x:c>
+      <x:c r="B28" s="61" t="n">
+        <x:v>105.995</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>Note 14 p.74: https://www.hkexnews.hk/listedco/listconews/sehk/2026/0924/2026092401584_c.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>RMB per USD</x:v>
+      </x:c>
+      <x:c r="B29" s="61" t="n">
+        <x:v>7.1</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>Model FX assumption retained</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1855,7 +1877,7 @@
       </x:c>
       <x:c r="B24" s="25" t="n">
         <x:f>B23+Assumptions!$B$7</x:f>
-        <x:v>3488.9488041686463</x:v>
+        <x:v>3474.01993092921</x:v>
       </x:c>
       <x:c r="C24" s="17"/>
       <x:c r="D24" s="17"/>
@@ -1878,7 +1900,7 @@
       </x:c>
       <x:c r="B25" s="25" t="n">
         <x:f>B24/Assumptions!$B$5</x:f>
-        <x:v>7.155525074799605</x:v>
+        <x:v>7.124907277635124</x:v>
       </x:c>
       <x:c r="C25" s="17"/>
       <x:c r="D25" s="17"/>
@@ -1901,7 +1923,7 @@
       </x:c>
       <x:c r="B26" s="25" t="n">
         <x:f>B25*Assumptions!$B$6</x:f>
-        <x:v>55.81309558343691</x:v>
+        <x:v>55.57427676555397</x:v>
       </x:c>
       <x:c r="C26" s="17"/>
       <x:c r="D26" s="17"/>
@@ -2835,7 +2857,7 @@
       </x:c>
       <x:c r="B24" s="25" t="n">
         <x:f>B23+Assumptions!$B$7</x:f>
-        <x:v>6362.5731451788715</x:v>
+        <x:v>6347.644271939435</x:v>
       </x:c>
       <x:c r="C24" s="17"/>
       <x:c r="D24" s="17"/>
@@ -2858,7 +2880,7 @@
       </x:c>
       <x:c r="B25" s="25" t="n">
         <x:f>B24/Assumptions!$B$5</x:f>
-        <x:v>13.049074158433344</x:v>
+        <x:v>13.018456361268864</x:v>
       </x:c>
       <x:c r="C25" s="17"/>
       <x:c r="D25" s="17"/>
@@ -2881,7 +2903,7 @@
       </x:c>
       <x:c r="B26" s="25" t="n">
         <x:f>B25*Assumptions!$B$6</x:f>
-        <x:v>101.78277843578007</x:v>
+        <x:v>101.54395961789714</x:v>
       </x:c>
       <x:c r="C26" s="17"/>
       <x:c r="D26" s="17"/>
@@ -3815,7 +3837,7 @@
       </x:c>
       <x:c r="B24" s="25" t="n">
         <x:f>B23+Assumptions!$B$7</x:f>
-        <x:v>15932.46370335871</x:v>
+        <x:v>15917.534830119273</x:v>
       </x:c>
       <x:c r="C24" s="17"/>
       <x:c r="D24" s="17"/>
@@ -3838,7 +3860,7 @@
       </x:c>
       <x:c r="B25" s="25" t="n">
         <x:f>B24/Assumptions!$B$5</x:f>
-        <x:v>32.67607234491455</x:v>
+        <x:v>32.64545454775008</x:v>
       </x:c>
       <x:c r="C25" s="17"/>
       <x:c r="D25" s="17"/>
@@ -3861,7 +3883,7 @@
       </x:c>
       <x:c r="B26" s="25" t="n">
         <x:f>B25*Assumptions!$B$6</x:f>
-        <x:v>254.87336429033348</x:v>
+        <x:v>254.63454547245058</x:v>
       </x:c>
       <x:c r="C26" s="17"/>
       <x:c r="D26" s="17"/>
@@ -3934,11 +3956,11 @@
       </x:c>
       <x:c r="C3" s="14" t="n">
         <x:f>Bear!B24</x:f>
-        <x:v>3488.9488041686463</x:v>
+        <x:v>3474.01993092921</x:v>
       </x:c>
       <x:c r="D3" s="14" t="n">
         <x:f>Bear!B26</x:f>
-        <x:v>55.81309558343691</x:v>
+        <x:v>55.57427676555397</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -3952,11 +3974,11 @@
       </x:c>
       <x:c r="C4" s="14" t="n">
         <x:f>Base!B24</x:f>
-        <x:v>6362.5731451788715</x:v>
+        <x:v>6347.644271939435</x:v>
       </x:c>
       <x:c r="D4" s="14" t="n">
         <x:f>Base!B26</x:f>
-        <x:v>101.78277843578007</x:v>
+        <x:v>101.54395961789714</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -3970,11 +3992,11 @@
       </x:c>
       <x:c r="C5" s="14" t="n">
         <x:f>Bull!B24</x:f>
-        <x:v>15932.46370335871</x:v>
+        <x:v>15917.534830119273</x:v>
       </x:c>
       <x:c r="D5" s="14" t="n">
         <x:f>Bull!B26</x:f>
-        <x:v>254.87336429033348</x:v>
+        <x:v>254.63454547245058</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -3986,11 +4008,11 @@
       <x:c r="B6" s="36"/>
       <x:c r="C6" s="37" t="n">
         <x:f>SUMPRODUCT(B3:B5,C3:C5)/SUM(B3:B5)</x:f>
-        <x:v>7270.782737461261</x:v>
+        <x:v>7255.853864221825</x:v>
       </x:c>
       <x:c r="D6" s="37" t="n">
         <x:f>SUMPRODUCT(B3:B5,D3:D5)/SUM(B3:B5)</x:f>
-        <x:v>116.31150660837065</x:v>
+        <x:v>116.07268779048772</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -4001,7 +4023,7 @@
       </x:c>
       <x:c r="B7" s="14" t="n">
         <x:f>Assumptions!B9</x:f>
-        <x:v>780</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="C7" s="6"/>
       <x:c r="D7" s="6"/>
@@ -4014,7 +4036,7 @@
       </x:c>
       <x:c r="B8" s="12" t="n">
         <x:f>D6/B7</x:f>
-        <x:v>0.14911731616457777</x:v>
+        <x:v>0.18108063617860798</x:v>
       </x:c>
       <x:c r="C8" s="6"/>
       <x:c r="D8" s="6"/>
@@ -4027,7 +4049,7 @@
       </x:c>
       <x:c r="B9" s="31" t="n">
         <x:f>(Assumptions!B9*Assumptions!B5/Assumptions!B6)/Assumptions!B12</x:f>
-        <x:v>232.76007026083917</x:v>
+        <x:v>191.28103209897168</x:v>
       </x:c>
       <x:c r="C9" s="6"/>
       <x:c r="D9" s="6"/>
@@ -4146,7 +4168,7 @@
         </x:is>
       </x:c>
       <x:c r="D2" s="44" t="str">
-        <x:v>2026-09-18</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="E2" s="45" t="inlineStr">
         <x:is>
@@ -4154,7 +4176,7 @@
         </x:is>
       </x:c>
       <x:c r="F2" s="51" t="n">
-        <x:v>48.75880900000001</x:v>
+        <x:v>40.06973919102565</x:v>
       </x:c>
       <x:c r="G2" s="51" t="n">
         <x:v>0.209480985915493</x:v>
@@ -4185,7 +4207,7 @@
       </x:c>
       <x:c r="N2" s="55" t="n">
         <x:f>F2/G2</x:f>
-        <x:v>232.76007026083914</x:v>
+        <x:v>191.28103209897168</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
@@ -4205,7 +4227,7 @@
         </x:is>
       </x:c>
       <x:c r="D3" s="46" t="str">
-        <x:v>2026-09-18</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="E3" s="47" t="inlineStr">
         <x:is>
@@ -4213,7 +4235,7 @@
         </x:is>
       </x:c>
       <x:c r="F3" s="52" t="n">
-        <x:v>13.566449071633238</x:v>
+        <x:v>11.202394579942691</x:v>
       </x:c>
       <x:c r="G3" s="52" t="n">
         <x:v>0.165182</x:v>
@@ -4240,11 +4262,11 @@
         </x:is>
       </x:c>
       <x:c r="M3" s="47" t="str">
-        <x:v>Closest listed foundation-model peer; public-market LTM multiple is shown separately from private transaction references. Price refreshed to 2026-09-11; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-17; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-18; share-count and FX basis carried forward from the 2026-08-31 snapshot.</x:v>
+        <x:v>Closest listed foundation-model peer; public-market LTM multiple is shown separately from private transaction references. Price refreshed to 2026-09-11; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-17; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-18; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-24; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-30; share-count and FX basis carried forward from the 2026-08-31 snapshot.</x:v>
       </x:c>
       <x:c r="N3" s="56" t="n">
         <x:f>F3/G3</x:f>
-        <x:v>82.13031124234625</x:v>
+        <x:v>67.81849462981857</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
@@ -4367,10 +4389,8 @@
           <x:t xml:space="preserve">https://www.anthropic.com/news/series-h</x:t>
         </x:is>
       </x:c>
-      <x:c r="M5" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Private frontier-lab transaction reference with valuation and revenue disclosed together by the company.</x:t>
-        </x:is>
+      <x:c r="M5" s="47" t="str">
+        <x:v>Private frontier-lab transaction reference with valuation and revenue disclosed together by the company. The September IPO target and 2028 forecast are separately modelled in ANTHROPIC_COMPARISON.md; excluded from the completed-deal range.</x:v>
       </x:c>
       <x:c r="N5" s="56" t="n">
         <x:f>F5/G5</x:f>
@@ -4589,7 +4609,7 @@
         </x:is>
       </x:c>
       <x:c r="D9" s="48" t="str">
-        <x:v>2026-09-18</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="E9" s="49" t="inlineStr">
         <x:is>
@@ -4597,7 +4617,7 @@
         </x:is>
       </x:c>
       <x:c r="F9" s="53" t="n">
-        <x:v>12.025440898837209</x:v>
+        <x:v>9.633932263372092</x:v>
       </x:c>
       <x:c r="G9" s="53" t="n">
         <x:v>0.459773</x:v>
@@ -4624,11 +4644,11 @@
         </x:is>
       </x:c>
       <x:c r="M9" s="49" t="str">
-        <x:v>Decision-intelligence and project-delivery model with a short trading history; contextual only. Price refreshed to 2026-09-11; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-18; share-count and FX basis carried forward from the 2026-08-31 snapshot.</x:v>
+        <x:v>Decision-intelligence and project-delivery model with a short trading history; contextual only. Price refreshed to 2026-09-11; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-18; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-24; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-30; share-count and FX basis carried forward from the 2026-08-31 snapshot.</x:v>
       </x:c>
       <x:c r="N9" s="57" t="n">
         <x:f>F9/G9</x:f>
-        <x:v>26.15516983128024</x:v>
+        <x:v>20.95367118854759</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -4844,7 +4864,7 @@
         <x:v>Market date</x:v>
       </x:c>
       <x:c r="B1" s="28" t="str">
-        <x:v>2026-09-18</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -4852,7 +4872,7 @@
         <x:v>Market price (HK$)</x:v>
       </x:c>
       <x:c r="B2" s="14" t="n">
-        <x:v>780</x:v>
+        <x:v>641</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4860,7 +4880,7 @@
         <x:v>Market equity value (US$m)</x:v>
       </x:c>
       <x:c r="B3" s="14" t="n">
-        <x:v>48758.8</x:v>
+        <x:v>40069.7</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -4868,7 +4888,7 @@
         <x:v>Market equity value / LTM revenue</x:v>
       </x:c>
       <x:c r="B4" s="14" t="n">
-        <x:v>232.8</x:v>
+        <x:v>191.3</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -4876,7 +4896,7 @@
         <x:v>Bear per share (HK$)</x:v>
       </x:c>
       <x:c r="B5" s="14" t="n">
-        <x:v>55.8</x:v>
+        <x:v>55.6</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -4884,7 +4904,7 @@
         <x:v>Base per share (HK$)</x:v>
       </x:c>
       <x:c r="B6" s="14" t="n">
-        <x:v>101.8</x:v>
+        <x:v>101.5</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -4892,7 +4912,7 @@
         <x:v>Bull per share (HK$)</x:v>
       </x:c>
       <x:c r="B7" s="14" t="n">
-        <x:v>254.9</x:v>
+        <x:v>254.6</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -4900,7 +4920,7 @@
         <x:v>Probability-weighted equity (US$m)</x:v>
       </x:c>
       <x:c r="B8" s="14" t="n">
-        <x:v>7270.8</x:v>
+        <x:v>7255.9</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4908,7 +4928,7 @@
         <x:v>Probability-weighted per share (HK$)</x:v>
       </x:c>
       <x:c r="B9" s="14" t="n">
-        <x:v>116.3</x:v>
+        <x:v>116.1</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -4916,7 +4936,7 @@
         <x:v>DCF value as % of market</x:v>
       </x:c>
       <x:c r="B10" s="12" t="n">
-        <x:v>0.1491</x:v>
+        <x:v>0.1811</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Update Zhipu valuation through October 9 and integrate Anthropic materials
</commit_message>
<xml_diff>
--- a/model/valuation_model.xlsx
+++ b/model/valuation_model.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="Ra8b8c6446c454431"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bear" sheetId="2" r:id="R9d9269088fc449f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="3" r:id="R13f6ad149da64d7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull" sheetId="4" r:id="Refd2ecf0c1354b8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="R84d50c8ccc0a40c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Comps" sheetId="6" r:id="Refda385eb32745b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="7" r:id="R81ac4e99dcdd4e31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="R7b694aa22b1a454a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bear" sheetId="2" r:id="Rf4e3f9595bbe411f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="3" r:id="R1a664a4b82c14b54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull" sheetId="4" r:id="R06949c65513544da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="Ree1f15c7091b4cff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Comps" sheetId="6" r:id="R2101c120e05a4b90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="7" r:id="R986283f8d4f84f64"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -669,7 +669,9 @@
       <x:c r="B5" s="13" t="n">
         <x:v>487.58809</x:v>
       </x:c>
-      <x:c r="C5" s="11"/>
+      <x:c r="C5" s="11" t="str">
+        <x:v>September monthly return (2 Oct): 263,059,605 H + 224,528,485 unlisted shares; awards unvested. https://www1.hkexnews.hk/listedco/listconews/sehk/2026/1002/2026100201832_c.pdf</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="6" t="inlineStr">
@@ -703,7 +705,7 @@
         </x:is>
       </x:c>
       <x:c r="B8" s="14" t="str">
-        <x:v>2026-09-30</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
       <x:c r="C8" s="11" t="inlineStr">
         <x:is>
@@ -718,7 +720,7 @@
         </x:is>
       </x:c>
       <x:c r="B9" s="14" t="n">
-        <x:v>641</x:v>
+        <x:v>641.5</x:v>
       </x:c>
       <x:c r="C9" s="11"/>
     </x:row>
@@ -4023,7 +4025,7 @@
       </x:c>
       <x:c r="B7" s="14" t="n">
         <x:f>Assumptions!B9</x:f>
-        <x:v>641</x:v>
+        <x:v>641.5</x:v>
       </x:c>
       <x:c r="C7" s="6"/>
       <x:c r="D7" s="6"/>
@@ -4036,7 +4038,7 @@
       </x:c>
       <x:c r="B8" s="12" t="n">
         <x:f>D6/B7</x:f>
-        <x:v>0.18108063617860798</x:v>
+        <x:v>0.18093949772484447</x:v>
       </x:c>
       <x:c r="C8" s="6"/>
       <x:c r="D8" s="6"/>
@@ -4049,7 +4051,7 @@
       </x:c>
       <x:c r="B9" s="31" t="n">
         <x:f>(Assumptions!B9*Assumptions!B5/Assumptions!B6)/Assumptions!B12</x:f>
-        <x:v>191.28103209897168</x:v>
+        <x:v>191.43023727221578</x:v>
       </x:c>
       <x:c r="C9" s="6"/>
       <x:c r="D9" s="6"/>
@@ -4152,44 +4154,32 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
-      <x:c r="A2" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Zhipu</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B2" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">02513.HK</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C2" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">core_frontier</x:t>
-        </x:is>
+      <x:c r="A2" s="44" t="str">
+        <x:v>Zhipu</x:v>
+      </x:c>
+      <x:c r="B2" s="44" t="str">
+        <x:v>02513.HK</x:v>
+      </x:c>
+      <x:c r="C2" s="44" t="str">
+        <x:v>core_frontier</x:v>
       </x:c>
       <x:c r="D2" s="44" t="str">
-        <x:v>2026-09-30</x:v>
-      </x:c>
-      <x:c r="E2" s="45" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">public market equity value</x:t>
-        </x:is>
+        <x:v>2026-10-09</x:v>
+      </x:c>
+      <x:c r="E2" s="45" t="str">
+        <x:v>public market equity value</x:v>
       </x:c>
       <x:c r="F2" s="51" t="n">
-        <x:v>40.06973919102565</x:v>
+        <x:v>40.100994837820515</x:v>
       </x:c>
       <x:c r="G2" s="51" t="n">
-        <x:v>0.209480985915493</x:v>
-      </x:c>
-      <x:c r="H2" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">USD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I2" s="45" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">LTM through 2026H1</x:t>
-        </x:is>
+        <x:v>0.20948098591549297</x:v>
+      </x:c>
+      <x:c r="H2" s="44" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I2" s="45" t="str">
+        <x:v>LTM through 2026H1</x:v>
       </x:c>
       <x:c r="J2" s="44" t="n">
         <x:v>0</x:v>
@@ -4197,58 +4187,44 @@
       <x:c r="K2" s="45" t="str">
         <x:v>https://web.ifzq.gtimg.cn/appstock/app/hkfqkline/get</x:v>
       </x:c>
-      <x:c r="L2" s="45" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0831/2026083101539.pdf</x:t>
-        </x:is>
+      <x:c r="L2" s="45" t="str">
+        <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0831/2026083101539.pdf</x:v>
       </x:c>
       <x:c r="M2" s="45" t="str">
         <x:v>Subject company; equity value is refreshed from the local market file and post-placement share count; LTM revenue is FY2025 less H1 2025 plus H1 2026 and translated at USD/CNY 7.1.</x:v>
       </x:c>
       <x:c r="N2" s="55" t="n">
         <x:f>F2/G2</x:f>
-        <x:v>191.28103209897168</x:v>
+        <x:v>191.4302372722158</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
-      <x:c r="A3" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MiniMax</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">00100.HK</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">core_frontier</x:t>
-        </x:is>
+      <x:c r="A3" s="46" t="str">
+        <x:v>MiniMax</x:v>
+      </x:c>
+      <x:c r="B3" s="46" t="str">
+        <x:v>00100.HK</x:v>
+      </x:c>
+      <x:c r="C3" s="46" t="str">
+        <x:v>core_frontier</x:v>
       </x:c>
       <x:c r="D3" s="46" t="str">
-        <x:v>2026-09-30</x:v>
-      </x:c>
-      <x:c r="E3" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">public market equity value</x:t>
-        </x:is>
+        <x:v>2026-10-09</x:v>
+      </x:c>
+      <x:c r="E3" s="47" t="str">
+        <x:v>public market equity value</x:v>
       </x:c>
       <x:c r="F3" s="52" t="n">
-        <x:v>11.202394579942691</x:v>
+        <x:v>9.536810733524351</x:v>
       </x:c>
       <x:c r="G3" s="52" t="n">
         <x:v>0.165182</x:v>
       </x:c>
-      <x:c r="H3" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">USD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I3" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">LTM through 2026H1</x:t>
-        </x:is>
+      <x:c r="H3" s="46" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I3" s="47" t="str">
+        <x:v>LTM through 2026H1</x:v>
       </x:c>
       <x:c r="J3" s="46" t="n">
         <x:v>0</x:v>
@@ -4256,44 +4232,32 @@
       <x:c r="K3" s="47" t="str">
         <x:v>https://web.ifzq.gtimg.cn/appstock/app/hkfqkline/get</x:v>
       </x:c>
-      <x:c r="L3" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0826/2026082600680.pdf</x:t>
-        </x:is>
+      <x:c r="L3" s="47" t="str">
+        <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0826/2026082600680.pdf</x:v>
       </x:c>
       <x:c r="M3" s="47" t="str">
-        <x:v>Closest listed foundation-model peer; public-market LTM multiple is shown separately from private transaction references. Price refreshed to 2026-09-11; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-17; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-18; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-24; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-30; share-count and FX basis carried forward from the 2026-08-31 snapshot.</x:v>
+        <x:v>Closest listed foundation-model peer; public-market LTM multiple is shown separately from private transaction references. Price refreshed to 2026-10-09; share-count and FX basis carried forward from 2026-08-31.</x:v>
       </x:c>
       <x:c r="N3" s="56" t="n">
         <x:f>F3/G3</x:f>
-        <x:v>67.81849462981857</x:v>
+        <x:v>57.735169289174074</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
-      <x:c r="A4" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">OpenAI</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">private</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">core_frontier</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D4" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-03-31</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">post-money financing</x:t>
-        </x:is>
+      <x:c r="A4" s="46" t="str">
+        <x:v>OpenAI</x:v>
+      </x:c>
+      <x:c r="B4" s="46" t="str">
+        <x:v>private</x:v>
+      </x:c>
+      <x:c r="C4" s="46" t="str">
+        <x:v>core_frontier</x:v>
+      </x:c>
+      <x:c r="D4" s="46" t="str">
+        <x:v>2026-03-31</x:v>
+      </x:c>
+      <x:c r="E4" s="47" t="str">
+        <x:v>post-money financing</x:v>
       </x:c>
       <x:c r="F4" s="52" t="n">
         <x:v>852</x:v>
@@ -4301,33 +4265,23 @@
       <x:c r="G4" s="52" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="H4" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">USD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I4" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">annualized revenue at February 2026</x:t>
-        </x:is>
+      <x:c r="H4" s="46" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I4" s="47" t="str">
+        <x:v>annualized revenue at February 2026</x:v>
       </x:c>
       <x:c r="J4" s="46" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K4" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://openai.com/index/accelerating-the-next-phase-ai/</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L4" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://finance.yahoo.com/news/openai-tops-25-billion-annualized-033836274.html</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M4" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Private frontier-lab transaction reference; revenue was reported by Reuters and was not independently verified.</x:t>
-        </x:is>
+      <x:c r="K4" s="47" t="str">
+        <x:v>https://openai.com/index/accelerating-the-next-phase-ai/</x:v>
+      </x:c>
+      <x:c r="L4" s="47" t="str">
+        <x:v>https://finance.yahoo.com/news/openai-tops-25-billion-annualized-033836274.html</x:v>
+      </x:c>
+      <x:c r="M4" s="47" t="str">
+        <x:v>Private frontier-lab transaction reference; revenue was reported by Reuters and was not independently verified.</x:v>
       </x:c>
       <x:c r="N4" s="56" t="n">
         <x:f>F4/G4</x:f>
@@ -4335,30 +4289,20 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
-      <x:c r="A5" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Anthropic</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">private</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C5" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">core_frontier</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D5" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-05-28</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E5" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">post-money financing</x:t>
-        </x:is>
+      <x:c r="A5" s="46" t="str">
+        <x:v>Anthropic</x:v>
+      </x:c>
+      <x:c r="B5" s="46" t="str">
+        <x:v>private</x:v>
+      </x:c>
+      <x:c r="C5" s="46" t="str">
+        <x:v>core_frontier</x:v>
+      </x:c>
+      <x:c r="D5" s="46" t="str">
+        <x:v>2026-05-28</x:v>
+      </x:c>
+      <x:c r="E5" s="47" t="str">
+        <x:v>post-money financing</x:v>
       </x:c>
       <x:c r="F5" s="52" t="n">
         <x:v>965</x:v>
@@ -4366,28 +4310,20 @@
       <x:c r="G5" s="52" t="n">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="H5" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">USD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I5" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">annualized revenue at May 2026</x:t>
-        </x:is>
+      <x:c r="H5" s="46" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I5" s="47" t="str">
+        <x:v>annualized revenue at May 2026</x:v>
       </x:c>
       <x:c r="J5" s="46" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K5" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.anthropic.com/news/series-h</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L5" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.anthropic.com/news/series-h</x:t>
-        </x:is>
+      <x:c r="K5" s="47" t="str">
+        <x:v>https://www.anthropic.com/news/series-h</x:v>
+      </x:c>
+      <x:c r="L5" s="47" t="str">
+        <x:v>https://www.anthropic.com/news/series-h</x:v>
       </x:c>
       <x:c r="M5" s="47" t="str">
         <x:v>Private frontier-lab transaction reference with valuation and revenue disclosed together by the company. The September IPO target and 2028 forecast are separately modelled in ANTHROPIC_COMPARISON.md; excluded from the completed-deal range.</x:v>
@@ -4398,30 +4334,20 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
-      <x:c r="A6" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Mistral</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">private</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C6" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">core_frontier</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D6" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2025-09-09</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E6" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">post-money financing</x:t>
-        </x:is>
+      <x:c r="A6" s="46" t="str">
+        <x:v>Mistral</x:v>
+      </x:c>
+      <x:c r="B6" s="46" t="str">
+        <x:v>private</x:v>
+      </x:c>
+      <x:c r="C6" s="46" t="str">
+        <x:v>core_frontier</x:v>
+      </x:c>
+      <x:c r="D6" s="46" t="str">
+        <x:v>2025-09-09</x:v>
+      </x:c>
+      <x:c r="E6" s="47" t="str">
+        <x:v>post-money financing</x:v>
       </x:c>
       <x:c r="F6" s="52" t="n">
         <x:v>11.7</x:v>
@@ -4429,33 +4355,23 @@
       <x:c r="G6" s="52" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="H6" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">EUR</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I6" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">annualized revenue at September 2025</x:t>
-        </x:is>
+      <x:c r="H6" s="46" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="I6" s="47" t="str">
+        <x:v>annualized revenue at September 2025</x:v>
       </x:c>
       <x:c r="J6" s="46" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K6" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://mistral.ai/news/mistral-ai-raises-1-7-b-to-accelerate-technological-progress-with-ai/</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L6" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.lemonde.fr/economie/article/2025/09/26/mistral-ai-incarnation-de-l-intelligence-artificielle_6643087_3234.html</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M6" s="47" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Older private frontier-lab reference; included in the private transaction range but dated separately.</x:t>
-        </x:is>
+      <x:c r="K6" s="47" t="str">
+        <x:v>https://mistral.ai/news/mistral-ai-raises-1-7-b-to-accelerate-technological-progress-with-ai/</x:v>
+      </x:c>
+      <x:c r="L6" s="47" t="str">
+        <x:v>https://www.lemonde.fr/economie/article/2025/09/26/mistral-ai-incarnation-de-l-intelligence-artificielle_6643087_3234.html</x:v>
+      </x:c>
+      <x:c r="M6" s="47" t="str">
+        <x:v>Older private frontier-lab reference; included in the private transaction range but dated separately.</x:v>
       </x:c>
       <x:c r="N6" s="56" t="n">
         <x:f>F6/G6</x:f>
@@ -4463,30 +4379,20 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
-      <x:c r="A7" s="48" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SenseTime</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B7" s="48" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">00020.HK</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C7" s="48" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">hk_adjacent</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D7" s="48" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-31</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E7" s="49" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">implied total equity value</x:t>
-        </x:is>
+      <x:c r="A7" s="48" t="str">
+        <x:v>SenseTime</x:v>
+      </x:c>
+      <x:c r="B7" s="48" t="str">
+        <x:v>00020.HK</x:v>
+      </x:c>
+      <x:c r="C7" s="48" t="str">
+        <x:v>hk_adjacent</x:v>
+      </x:c>
+      <x:c r="D7" s="48" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="E7" s="49" t="str">
+        <x:v>implied total equity value</x:v>
       </x:c>
       <x:c r="F7" s="53" t="n">
         <x:v>52.58377</x:v>
@@ -4494,33 +4400,23 @@
       <x:c r="G7" s="53" t="n">
         <x:v>5.567388</x:v>
       </x:c>
-      <x:c r="H7" s="48" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">CNY</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I7" s="49" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">LTM through 2026H1</x:t>
-        </x:is>
+      <x:c r="H7" s="48" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="I7" s="49" t="str">
+        <x:v>LTM through 2026H1</x:v>
       </x:c>
       <x:c r="J7" s="48" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K7" s="49" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.hkex.com.hk/chi/stat/smstat/dayquot/d260831c.htm</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L7" s="49" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0826/2026082600408.pdf</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M7" s="49" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Adjacent Hong Kong AI platform; mixed computer-vision generative-AI and solution revenue makes it contextual only.</x:t>
-        </x:is>
+      <x:c r="K7" s="49" t="str">
+        <x:v>https://www.hkex.com.hk/chi/stat/smstat/dayquot/d260831c.htm</x:v>
+      </x:c>
+      <x:c r="L7" s="49" t="str">
+        <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0826/2026082600408.pdf</x:v>
+      </x:c>
+      <x:c r="M7" s="49" t="str">
+        <x:v>Adjacent Hong Kong AI platform; mixed computer-vision generative-AI and solution revenue makes it contextual only.</x:v>
       </x:c>
       <x:c r="N7" s="57" t="n">
         <x:f>F7/G7</x:f>
@@ -4528,64 +4424,44 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
-      <x:c r="A8" s="48" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Phancy</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B8" s="48" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">06682.HK</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C8" s="48" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">hk_adjacent</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D8" s="48" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-31</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E8" s="49" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">implied total equity value</x:t>
-        </x:is>
+      <x:c r="A8" s="48" t="str">
+        <x:v>Phancy</x:v>
+      </x:c>
+      <x:c r="B8" s="48" t="str">
+        <x:v>06682.HK</x:v>
+      </x:c>
+      <x:c r="C8" s="48" t="str">
+        <x:v>hk_adjacent</x:v>
+      </x:c>
+      <x:c r="D8" s="48" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="E8" s="49" t="str">
+        <x:v>implied total equity value</x:v>
       </x:c>
       <x:c r="F8" s="53" t="n">
         <x:v>13.500771</x:v>
       </x:c>
       <x:c r="G8" s="53" t="n">
-        <x:v>8.274082999999999</x:v>
-      </x:c>
-      <x:c r="H8" s="48" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">CNY</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I8" s="49" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">LTM through 2026H1</x:t>
-        </x:is>
+        <x:v>8.274083</x:v>
+      </x:c>
+      <x:c r="H8" s="48" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="I8" s="49" t="str">
+        <x:v>LTM through 2026H1</x:v>
       </x:c>
       <x:c r="J8" s="48" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K8" s="49" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.hkex.com.hk/chi/stat/smstat/dayquot/d260831c.htm</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L8" s="49" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0820/2026082000357.pdf</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M8" s="49" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Enterprise AI platform and agentic services with a different revenue and margin mix; contextual only.</x:t>
-        </x:is>
+      <x:c r="K8" s="49" t="str">
+        <x:v>https://www.hkex.com.hk/chi/stat/smstat/dayquot/d260831c.htm</x:v>
+      </x:c>
+      <x:c r="L8" s="49" t="str">
+        <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0820/2026082000357.pdf</x:v>
+      </x:c>
+      <x:c r="M8" s="49" t="str">
+        <x:v>Enterprise AI platform and agentic services with a different revenue and margin mix; contextual only.</x:v>
       </x:c>
       <x:c r="N8" s="57" t="n">
         <x:f>F8/G8</x:f>
@@ -4593,44 +4469,32 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
-      <x:c r="A9" s="48" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Wenge AI</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B9" s="48" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">01956.HK</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C9" s="48" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">hk_adjacent</x:t>
-        </x:is>
+      <x:c r="A9" s="48" t="str">
+        <x:v>Wenge AI</x:v>
+      </x:c>
+      <x:c r="B9" s="48" t="str">
+        <x:v>01956.HK</x:v>
+      </x:c>
+      <x:c r="C9" s="48" t="str">
+        <x:v>hk_adjacent</x:v>
       </x:c>
       <x:c r="D9" s="48" t="str">
-        <x:v>2026-09-30</x:v>
-      </x:c>
-      <x:c r="E9" s="49" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">implied total equity value</x:t>
-        </x:is>
+        <x:v>2026-10-09</x:v>
+      </x:c>
+      <x:c r="E9" s="49" t="str">
+        <x:v>implied total equity value</x:v>
       </x:c>
       <x:c r="F9" s="53" t="n">
-        <x:v>9.633932263372092</x:v>
+        <x:v>9.596211306976745</x:v>
       </x:c>
       <x:c r="G9" s="53" t="n">
         <x:v>0.459773</x:v>
       </x:c>
-      <x:c r="H9" s="48" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">CNY</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I9" s="49" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">LTM through 2026H1</x:t>
-        </x:is>
+      <x:c r="H9" s="48" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="I9" s="49" t="str">
+        <x:v>LTM through 2026H1</x:v>
       </x:c>
       <x:c r="J9" s="48" t="n">
         <x:v>0</x:v>
@@ -4638,44 +4502,32 @@
       <x:c r="K9" s="49" t="str">
         <x:v>https://web.ifzq.gtimg.cn/appstock/app/hkfqkline/get</x:v>
       </x:c>
-      <x:c r="L9" s="49" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0825/2026082500959.pdf</x:t>
-        </x:is>
+      <x:c r="L9" s="49" t="str">
+        <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0825/2026082500959.pdf</x:v>
       </x:c>
       <x:c r="M9" s="49" t="str">
-        <x:v>Decision-intelligence and project-delivery model with a short trading history; contextual only. Price refreshed to 2026-09-11; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-18; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-24; share-count and FX basis carried forward from the 2026-08-31 snapshot. Price refreshed to 2026-09-30; share-count and FX basis carried forward from the 2026-08-31 snapshot.</x:v>
+        <x:v>Decision-intelligence and project-delivery model with a short trading history; contextual only. Price refreshed to 2026-10-09; share-count and FX basis carried forward from 2026-08-31.</x:v>
       </x:c>
       <x:c r="N9" s="57" t="n">
         <x:f>F9/G9</x:f>
-        <x:v>20.95367118854759</x:v>
+        <x:v>20.87162862320481</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
-      <x:c r="A10" s="32" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Palantir</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B10" s="32" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">PLTR</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C10" s="32" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">commercialization_reference</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D10" s="32" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-31</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E10" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">public market equity value</x:t>
-        </x:is>
+      <x:c r="A10" s="32" t="str">
+        <x:v>Palantir</x:v>
+      </x:c>
+      <x:c r="B10" s="32" t="str">
+        <x:v>PLTR</x:v>
+      </x:c>
+      <x:c r="C10" s="32" t="str">
+        <x:v>commercialization_reference</x:v>
+      </x:c>
+      <x:c r="D10" s="32" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="E10" s="50" t="str">
+        <x:v>public market equity value</x:v>
       </x:c>
       <x:c r="F10" s="54" t="n">
         <x:v>447.856263</x:v>
@@ -4683,33 +4535,23 @@
       <x:c r="G10" s="54" t="n">
         <x:v>4.475446</x:v>
       </x:c>
-      <x:c r="H10" s="32" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">USD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I10" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FY2025 revenue</x:t>
-        </x:is>
+      <x:c r="H10" s="32" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I10" s="50" t="str">
+        <x:v>FY2025 revenue</x:v>
       </x:c>
       <x:c r="J10" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K10" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.gurufocus.com/stock/PLTR/data/market-cap</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L10" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.sec.gov/Archives/edgar/data/1321655/000132165526000011/pltr-20251231.htm</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M10" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Mature AI software commercialization reference; not a frontier-model laboratory.</x:t>
-        </x:is>
+      <x:c r="K10" s="50" t="str">
+        <x:v>https://www.gurufocus.com/stock/PLTR/data/market-cap</x:v>
+      </x:c>
+      <x:c r="L10" s="50" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1321655/000132165526000011/pltr-20251231.htm</x:v>
+      </x:c>
+      <x:c r="M10" s="50" t="str">
+        <x:v>Mature AI software commercialization reference; not a frontier-model laboratory.</x:v>
       </x:c>
       <x:c r="N10" s="58" t="n">
         <x:f>F10/G10</x:f>
@@ -4717,30 +4559,20 @@
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
-      <x:c r="A11" s="32" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cloudflare</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B11" s="32" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">NET</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C11" s="32" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">commercialization_reference</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D11" s="32" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-31</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E11" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">public market equity value</x:t>
-        </x:is>
+      <x:c r="A11" s="32" t="str">
+        <x:v>Cloudflare</x:v>
+      </x:c>
+      <x:c r="B11" s="32" t="str">
+        <x:v>NET</x:v>
+      </x:c>
+      <x:c r="C11" s="32" t="str">
+        <x:v>commercialization_reference</x:v>
+      </x:c>
+      <x:c r="D11" s="32" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="E11" s="50" t="str">
+        <x:v>public market equity value</x:v>
       </x:c>
       <x:c r="F11" s="54" t="n">
         <x:v>108.259915</x:v>
@@ -4748,33 +4580,23 @@
       <x:c r="G11" s="54" t="n">
         <x:v>2.1679</x:v>
       </x:c>
-      <x:c r="H11" s="32" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">USD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I11" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FY2025 revenue</x:t>
-        </x:is>
+      <x:c r="H11" s="32" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I11" s="50" t="str">
+        <x:v>FY2025 revenue</x:v>
       </x:c>
       <x:c r="J11" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K11" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.tipranks.com/stocks/net/market-cap</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L11" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.cloudflare.com/press/press-releases/2026/cloudflare-announces-fourth-quarter-and-fiscal-year-2025-financial-results/</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M11" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Connectivity and inference-infrastructure reference; economics differ from a model laboratory.</x:t>
-        </x:is>
+      <x:c r="K11" s="50" t="str">
+        <x:v>https://www.tipranks.com/stocks/net/market-cap</x:v>
+      </x:c>
+      <x:c r="L11" s="50" t="str">
+        <x:v>https://www.cloudflare.com/press/press-releases/2026/cloudflare-announces-fourth-quarter-and-fiscal-year-2025-financial-results/</x:v>
+      </x:c>
+      <x:c r="M11" s="50" t="str">
+        <x:v>Connectivity and inference-infrastructure reference; economics differ from a model laboratory.</x:v>
       </x:c>
       <x:c r="N11" s="58" t="n">
         <x:f>F11/G11</x:f>
@@ -4782,30 +4604,20 @@
       </x:c>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
-      <x:c r="A12" s="32" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Snowflake</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B12" s="32" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SNOW</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C12" s="32" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">commercialization_reference</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D12" s="32" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-31</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E12" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">public market equity value</x:t>
-        </x:is>
+      <x:c r="A12" s="32" t="str">
+        <x:v>Snowflake</x:v>
+      </x:c>
+      <x:c r="B12" s="32" t="str">
+        <x:v>SNOW</x:v>
+      </x:c>
+      <x:c r="C12" s="32" t="str">
+        <x:v>commercialization_reference</x:v>
+      </x:c>
+      <x:c r="D12" s="32" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="E12" s="50" t="str">
+        <x:v>public market equity value</x:v>
       </x:c>
       <x:c r="F12" s="54" t="n">
         <x:v>114.87384</x:v>
@@ -4813,33 +4625,23 @@
       <x:c r="G12" s="54" t="n">
         <x:v>4.683946</x:v>
       </x:c>
-      <x:c r="H12" s="32" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">USD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I12" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FY2026 revenue</x:t>
-        </x:is>
+      <x:c r="H12" s="32" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="I12" s="50" t="str">
+        <x:v>FY2026 revenue</x:v>
       </x:c>
       <x:c r="J12" s="32" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K12" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://finance.yahoo.com/quote/SNOW/history/</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L12" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.sec.gov/Archives/edgar/data/1640147/000164014726000023/snowflake2026ars.pdf</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M12" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Data-cloud commercialization reference; not a direct foundation-model comparable.</x:t>
-        </x:is>
+      <x:c r="K12" s="50" t="str">
+        <x:v>https://finance.yahoo.com/quote/SNOW/history/</x:v>
+      </x:c>
+      <x:c r="L12" s="50" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/1640147/000164014726000023/snowflake2026ars.pdf</x:v>
+      </x:c>
+      <x:c r="M12" s="50" t="str">
+        <x:v>Data-cloud commercialization reference; not a direct foundation-model comparable.</x:v>
       </x:c>
       <x:c r="N12" s="58" t="n">
         <x:f>F12/G12</x:f>
@@ -4864,7 +4666,7 @@
         <x:v>Market date</x:v>
       </x:c>
       <x:c r="B1" s="28" t="str">
-        <x:v>2026-09-30</x:v>
+        <x:v>2026-10-09</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -4872,7 +4674,7 @@
         <x:v>Market price (HK$)</x:v>
       </x:c>
       <x:c r="B2" s="14" t="n">
-        <x:v>641</x:v>
+        <x:v>641.5</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4880,7 +4682,7 @@
         <x:v>Market equity value (US$m)</x:v>
       </x:c>
       <x:c r="B3" s="14" t="n">
-        <x:v>40069.7</x:v>
+        <x:v>40101</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -4888,7 +4690,7 @@
         <x:v>Market equity value / LTM revenue</x:v>
       </x:c>
       <x:c r="B4" s="14" t="n">
-        <x:v>191.3</x:v>
+        <x:v>191.4</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -4936,7 +4738,7 @@
         <x:v>DCF value as % of market</x:v>
       </x:c>
       <x:c r="B10" s="12" t="n">
-        <x:v>0.1811</x:v>
+        <x:v>0.1809</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Refresh valuation and reports through October 14; remove redundant logs
</commit_message>
<xml_diff>
--- a/model/valuation_model.xlsx
+++ b/model/valuation_model.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="R7b694aa22b1a454a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bear" sheetId="2" r:id="Rf4e3f9595bbe411f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="3" r:id="R1a664a4b82c14b54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull" sheetId="4" r:id="R06949c65513544da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="Ree1f15c7091b4cff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Comps" sheetId="6" r:id="R2101c120e05a4b90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="7" r:id="R986283f8d4f84f64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="R162172a2f7194036"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bear" sheetId="2" r:id="Rbca2de0c754f4a60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="3" r:id="R3b521c7225864735"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull" sheetId="4" r:id="R1e070cc8ce064966"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="R80a58e740b8d4c6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Comps" sheetId="6" r:id="Re0786eb5842d4035"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="7" r:id="R49e248e9259d40db"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -705,7 +705,7 @@
         </x:is>
       </x:c>
       <x:c r="B8" s="14" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-10-14</x:v>
       </x:c>
       <x:c r="C8" s="11" t="inlineStr">
         <x:is>
@@ -720,7 +720,7 @@
         </x:is>
       </x:c>
       <x:c r="B9" s="14" t="n">
-        <x:v>641.5</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="C9" s="11"/>
     </x:row>
@@ -4025,7 +4025,7 @@
       </x:c>
       <x:c r="B7" s="14" t="n">
         <x:f>Assumptions!B9</x:f>
-        <x:v>641.5</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="C7" s="6"/>
       <x:c r="D7" s="6"/>
@@ -4038,7 +4038,7 @@
       </x:c>
       <x:c r="B8" s="12" t="n">
         <x:f>D6/B7</x:f>
-        <x:v>0.18093949772484447</x:v>
+        <x:v>0.2029242793539995</x:v>
       </x:c>
       <x:c r="C8" s="6"/>
       <x:c r="D8" s="6"/>
@@ -4051,7 +4051,7 @@
       </x:c>
       <x:c r="B9" s="31" t="n">
         <x:f>(Assumptions!B9*Assumptions!B5/Assumptions!B6)/Assumptions!B12</x:f>
-        <x:v>191.43023727221578</x:v>
+        <x:v>170.69071819128206</x:v>
       </x:c>
       <x:c r="C9" s="6"/>
       <x:c r="D9" s="6"/>
@@ -4164,13 +4164,13 @@
         <x:v>core_frontier</x:v>
       </x:c>
       <x:c r="D2" s="44" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-10-14</x:v>
       </x:c>
       <x:c r="E2" s="45" t="str">
         <x:v>public market equity value</x:v>
       </x:c>
       <x:c r="F2" s="51" t="n">
-        <x:v>40.100994837820515</x:v>
+        <x:v>35.75645993333334</x:v>
       </x:c>
       <x:c r="G2" s="51" t="n">
         <x:v>0.20948098591549297</x:v>
@@ -4195,7 +4195,7 @@
       </x:c>
       <x:c r="N2" s="55" t="n">
         <x:f>F2/G2</x:f>
-        <x:v>191.4302372722158</x:v>
+        <x:v>170.69071819128206</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
@@ -4209,13 +4209,13 @@
         <x:v>core_frontier</x:v>
       </x:c>
       <x:c r="D3" s="46" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-10-14</x:v>
       </x:c>
       <x:c r="E3" s="47" t="str">
         <x:v>public market equity value</x:v>
       </x:c>
       <x:c r="F3" s="52" t="n">
-        <x:v>9.536810733524351</x:v>
+        <x:v>9.142801651575928</x:v>
       </x:c>
       <x:c r="G3" s="52" t="n">
         <x:v>0.165182</x:v>
@@ -4236,11 +4236,11 @@
         <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0826/2026082600680.pdf</x:v>
       </x:c>
       <x:c r="M3" s="47" t="str">
-        <x:v>Closest listed foundation-model peer; public-market LTM multiple is shown separately from private transaction references. Price refreshed to 2026-10-09; share-count and FX basis carried forward from 2026-08-31.</x:v>
+        <x:v>Closest listed foundation-model peer; public-market LTM multiple is shown separately from private transaction references. Price refreshed to 2026-10-14; share-count and FX basis carried forward from 2026-08-31.</x:v>
       </x:c>
       <x:c r="N3" s="56" t="n">
         <x:f>F3/G3</x:f>
-        <x:v>57.735169289174074</x:v>
+        <x:v>55.34986652041947</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
@@ -4389,13 +4389,13 @@
         <x:v>hk_adjacent</x:v>
       </x:c>
       <x:c r="D7" s="48" t="str">
-        <x:v>2026-08-31</x:v>
+        <x:v>2026-10-14</x:v>
       </x:c>
       <x:c r="E7" s="49" t="str">
         <x:v>implied total equity value</x:v>
       </x:c>
       <x:c r="F7" s="53" t="n">
-        <x:v>52.58377</x:v>
+        <x:v>43.45464326388889</x:v>
       </x:c>
       <x:c r="G7" s="53" t="n">
         <x:v>5.567388</x:v>
@@ -4410,17 +4410,17 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K7" s="49" t="str">
-        <x:v>https://www.hkex.com.hk/chi/stat/smstat/dayquot/d260831c.htm</x:v>
+        <x:v>https://web.ifzq.gtimg.cn/appstock/app/hkfqkline/get?param=hk00020%2Cday%2C2026-08-31%2C2026-10-14%2C640%2Cqfq</x:v>
       </x:c>
       <x:c r="L7" s="49" t="str">
         <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0826/2026082600408.pdf</x:v>
       </x:c>
       <x:c r="M7" s="49" t="str">
-        <x:v>Adjacent Hong Kong AI platform; mixed computer-vision generative-AI and solution revenue makes it contextual only.</x:v>
+        <x:v>Adjacent Hong Kong AI platform; mixed computer-vision generative-AI and solution revenue makes it contextual only. Price refreshed to 2026-10-14; August share-count and FX basis retained, not a newly verified market capitalization.</x:v>
       </x:c>
       <x:c r="N7" s="57" t="n">
         <x:f>F7/G7</x:f>
-        <x:v>9.444962341406779</x:v>
+        <x:v>7.8052119349125455</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
@@ -4434,13 +4434,13 @@
         <x:v>hk_adjacent</x:v>
       </x:c>
       <x:c r="D8" s="48" t="str">
-        <x:v>2026-08-31</x:v>
+        <x:v>2026-10-14</x:v>
       </x:c>
       <x:c r="E8" s="49" t="str">
         <x:v>implied total equity value</x:v>
       </x:c>
       <x:c r="F8" s="53" t="n">
-        <x:v>13.500771</x:v>
+        <x:v>11.621648698072804</x:v>
       </x:c>
       <x:c r="G8" s="53" t="n">
         <x:v>8.274083</x:v>
@@ -4455,17 +4455,17 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K8" s="49" t="str">
-        <x:v>https://www.hkex.com.hk/chi/stat/smstat/dayquot/d260831c.htm</x:v>
+        <x:v>https://web.ifzq.gtimg.cn/appstock/app/hkfqkline/get?param=hk06682%2Cday%2C2026-08-31%2C2026-10-14%2C640%2Cqfq</x:v>
       </x:c>
       <x:c r="L8" s="49" t="str">
         <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0820/2026082000357.pdf</x:v>
       </x:c>
       <x:c r="M8" s="49" t="str">
-        <x:v>Enterprise AI platform and agentic services with a different revenue and margin mix; contextual only.</x:v>
+        <x:v>Enterprise AI platform and agentic services with a different revenue and margin mix; contextual only. Price refreshed to 2026-10-14; August share-count and FX basis retained, not a newly verified market capitalization.</x:v>
       </x:c>
       <x:c r="N8" s="57" t="n">
         <x:f>F8/G8</x:f>
-        <x:v>1.6316939291036845</x:v>
+        <x:v>1.4045844957166618</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
@@ -4479,13 +4479,13 @@
         <x:v>hk_adjacent</x:v>
       </x:c>
       <x:c r="D9" s="48" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-10-14</x:v>
       </x:c>
       <x:c r="E9" s="49" t="str">
         <x:v>implied total equity value</x:v>
       </x:c>
       <x:c r="F9" s="53" t="n">
-        <x:v>9.596211306976745</x:v>
+        <x:v>9.332164612209302</x:v>
       </x:c>
       <x:c r="G9" s="53" t="n">
         <x:v>0.459773</x:v>
@@ -4506,11 +4506,11 @@
         <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0825/2026082500959.pdf</x:v>
       </x:c>
       <x:c r="M9" s="49" t="str">
-        <x:v>Decision-intelligence and project-delivery model with a short trading history; contextual only. Price refreshed to 2026-10-09; share-count and FX basis carried forward from 2026-08-31.</x:v>
+        <x:v>Decision-intelligence and project-delivery model with a short trading history; contextual only. Price refreshed to 2026-10-14; share-count and FX basis carried forward from 2026-08-31.</x:v>
       </x:c>
       <x:c r="N9" s="57" t="n">
         <x:f>F9/G9</x:f>
-        <x:v>20.87162862320481</x:v>
+        <x:v>20.297330665805305</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -4524,13 +4524,13 @@
         <x:v>commercialization_reference</x:v>
       </x:c>
       <x:c r="D10" s="32" t="str">
-        <x:v>2026-08-31</x:v>
+        <x:v>2026-10-14</x:v>
       </x:c>
       <x:c r="E10" s="50" t="str">
         <x:v>public market equity value</x:v>
       </x:c>
       <x:c r="F10" s="54" t="n">
-        <x:v>447.856263</x:v>
+        <x:v>482.9148586963561</x:v>
       </x:c>
       <x:c r="G10" s="54" t="n">
         <x:v>4.475446</x:v>
@@ -4545,17 +4545,17 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K10" s="50" t="str">
-        <x:v>https://www.gurufocus.com/stock/PLTR/data/market-cap</x:v>
+        <x:v>https://query1.finance.yahoo.com/v8/finance/chart/PLTR?period1=1788134400&amp;period2=1792022400&amp;interval=1d</x:v>
       </x:c>
       <x:c r="L10" s="50" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1321655/000132165526000011/pltr-20251231.htm</x:v>
       </x:c>
       <x:c r="M10" s="50" t="str">
-        <x:v>Mature AI software commercialization reference; not a frontier-model laboratory.</x:v>
+        <x:v>Mature AI software commercialization reference; not a frontier-model laboratory. Price refreshed to 2026-10-14; August share-count and FX basis retained, not a newly verified market capitalization.</x:v>
       </x:c>
       <x:c r="N10" s="58" t="n">
         <x:f>F10/G10</x:f>
-        <x:v>100.06963842262873</x:v>
+        <x:v>107.90318075480211</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -4569,13 +4569,13 @@
         <x:v>commercialization_reference</x:v>
       </x:c>
       <x:c r="D11" s="32" t="str">
-        <x:v>2026-08-31</x:v>
+        <x:v>2026-10-14</x:v>
       </x:c>
       <x:c r="E11" s="50" t="str">
         <x:v>public market equity value</x:v>
       </x:c>
       <x:c r="F11" s="54" t="n">
-        <x:v>108.259915</x:v>
+        <x:v>115.07960559798444</x:v>
       </x:c>
       <x:c r="G11" s="54" t="n">
         <x:v>2.1679</x:v>
@@ -4590,17 +4590,17 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K11" s="50" t="str">
-        <x:v>https://www.tipranks.com/stocks/net/market-cap</x:v>
+        <x:v>https://query1.finance.yahoo.com/v8/finance/chart/NET?period1=1788134400&amp;period2=1792022400&amp;interval=1d</x:v>
       </x:c>
       <x:c r="L11" s="50" t="str">
         <x:v>https://www.cloudflare.com/press/press-releases/2026/cloudflare-announces-fourth-quarter-and-fiscal-year-2025-financial-results/</x:v>
       </x:c>
       <x:c r="M11" s="50" t="str">
-        <x:v>Connectivity and inference-infrastructure reference; economics differ from a model laboratory.</x:v>
+        <x:v>Connectivity and inference-infrastructure reference; economics differ from a model laboratory. Price refreshed to 2026-10-14; August share-count and FX basis retained, not a newly verified market capitalization.</x:v>
       </x:c>
       <x:c r="N11" s="58" t="n">
         <x:f>F11/G11</x:f>
-        <x:v>49.93768854651968</x:v>
+        <x:v>53.08344739055512</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
@@ -4614,13 +4614,13 @@
         <x:v>commercialization_reference</x:v>
       </x:c>
       <x:c r="D12" s="32" t="str">
-        <x:v>2026-08-31</x:v>
+        <x:v>2026-10-14</x:v>
       </x:c>
       <x:c r="E12" s="50" t="str">
         <x:v>public market equity value</x:v>
       </x:c>
       <x:c r="F12" s="54" t="n">
-        <x:v>114.87384</x:v>
+        <x:v>116.13893013707728</x:v>
       </x:c>
       <x:c r="G12" s="54" t="n">
         <x:v>4.683946</x:v>
@@ -4635,17 +4635,17 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K12" s="50" t="str">
-        <x:v>https://finance.yahoo.com/quote/SNOW/history/</x:v>
+        <x:v>https://query1.finance.yahoo.com/v8/finance/chart/SNOW?period1=1788134400&amp;period2=1792022400&amp;interval=1d</x:v>
       </x:c>
       <x:c r="L12" s="50" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1640147/000164014726000023/snowflake2026ars.pdf</x:v>
       </x:c>
       <x:c r="M12" s="50" t="str">
-        <x:v>Data-cloud commercialization reference; not a direct foundation-model comparable.</x:v>
+        <x:v>Data-cloud commercialization reference; not a direct foundation-model comparable. Price refreshed to 2026-10-14; August share-count and FX basis retained, not a newly verified market capitalization.</x:v>
       </x:c>
       <x:c r="N12" s="58" t="n">
         <x:f>F12/G12</x:f>
-        <x:v>24.525013738416284</x:v>
+        <x:v>24.795104413474725</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4666,7 +4666,7 @@
         <x:v>Market date</x:v>
       </x:c>
       <x:c r="B1" s="28" t="str">
-        <x:v>2026-10-09</x:v>
+        <x:v>2026-10-14</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -4674,7 +4674,7 @@
         <x:v>Market price (HK$)</x:v>
       </x:c>
       <x:c r="B2" s="14" t="n">
-        <x:v>641.5</x:v>
+        <x:v>572</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4682,7 +4682,7 @@
         <x:v>Market equity value (US$m)</x:v>
       </x:c>
       <x:c r="B3" s="14" t="n">
-        <x:v>40101</x:v>
+        <x:v>35756.5</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -4690,7 +4690,7 @@
         <x:v>Market equity value / LTM revenue</x:v>
       </x:c>
       <x:c r="B4" s="14" t="n">
-        <x:v>191.4</x:v>
+        <x:v>170.7</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -4738,7 +4738,7 @@
         <x:v>DCF value as % of market</x:v>
       </x:c>
       <x:c r="B10" s="12" t="n">
-        <x:v>0.1809</x:v>
+        <x:v>0.2029</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
chore: refresh valuation research through 2026-10-30
Update observed HK and US prices, valuation inputs, event windows, workbook, figures, paper and slides. Ten core tests pass; output reconciliation passes with --ignore-word-limits. The paper remains 6711 text words, exceeding the original 5000-word submission limit.
</commit_message>
<xml_diff>
--- a/model/valuation_model.xlsx
+++ b/model/valuation_model.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="R37c2c3b2421c4fee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bear" sheetId="2" r:id="Rdf414f3ec44e4fba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="3" r:id="R89ded0c4b1fe4b19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull" sheetId="4" r:id="R44e074f68f194bd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="R906264b995a34724"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Comps" sheetId="6" r:id="R1630110c53484a55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="7" r:id="R8d76a9c8082c4c3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" r:id="Red12bc3bc6754e95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bear" sheetId="2" r:id="R32f63253c7364734"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="3" r:id="Ra94fc2cec2c74e82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bull" sheetId="4" r:id="Rf15a8cb8d75d4c93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" r:id="R0a7347fa45774f12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Comps" sheetId="6" r:id="R53aac2b96d6c4a16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="7" r:id="R6b3e991adfe84109"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -705,7 +705,7 @@
         </x:is>
       </x:c>
       <x:c r="B8" s="14" t="str">
-        <x:v>2026-10-23</x:v>
+        <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="C8" s="11" t="inlineStr">
         <x:is>
@@ -720,7 +720,7 @@
         </x:is>
       </x:c>
       <x:c r="B9" s="14" t="n">
-        <x:v>499</x:v>
+        <x:v>483.6</x:v>
       </x:c>
       <x:c r="C9" s="11"/>
     </x:row>
@@ -4025,7 +4025,7 @@
       </x:c>
       <x:c r="B7" s="14" t="n">
         <x:f>Assumptions!B9</x:f>
-        <x:v>499</x:v>
+        <x:v>483.6</x:v>
       </x:c>
       <x:c r="C7" s="6"/>
       <x:c r="D7" s="6"/>
@@ -4038,7 +4038,7 @@
       </x:c>
       <x:c r="B8" s="12" t="n">
         <x:f>D6/B7</x:f>
-        <x:v>0.23261059677452448</x:v>
+        <x:v>0.24001796482731125</x:v>
       </x:c>
       <x:c r="C8" s="6"/>
       <x:c r="D8" s="6"/>
@@ -4051,7 +4051,7 @@
       </x:c>
       <x:c r="B9" s="31" t="n">
         <x:f>(Assumptions!B9*Assumptions!B5/Assumptions!B6)/Assumptions!B12</x:f>
-        <x:v>148.9067628976394</x:v>
+        <x:v>144.31124356172026</x:v>
       </x:c>
       <x:c r="C9" s="6"/>
       <x:c r="D9" s="6"/>
@@ -4164,16 +4164,16 @@
         <x:v>core_frontier</x:v>
       </x:c>
       <x:c r="D2" s="44" t="str">
-        <x:v>2026-10-23</x:v>
+        <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="E2" s="45" t="str">
         <x:v>public market equity value</x:v>
       </x:c>
       <x:c r="F2" s="51" t="n">
-        <x:v>31.193135501282054</x:v>
+        <x:v>30.230462</x:v>
       </x:c>
       <x:c r="G2" s="51" t="n">
-        <x:v>0.20948098591549297</x:v>
+        <x:v>0.209481</x:v>
       </x:c>
       <x:c r="H2" s="44" t="str">
         <x:v>USD</x:v>
@@ -4195,7 +4195,7 @@
       </x:c>
       <x:c r="N2" s="55" t="n">
         <x:f>F2/G2</x:f>
-        <x:v>148.90676289763942</x:v>
+        <x:v>144.3112358638731</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
@@ -4209,13 +4209,13 @@
         <x:v>core_frontier</x:v>
       </x:c>
       <x:c r="D3" s="46" t="str">
-        <x:v>2026-10-23</x:v>
+        <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="E3" s="47" t="str">
         <x:v>public market equity value</x:v>
       </x:c>
       <x:c r="F3" s="52" t="n">
-        <x:v>8.399557246991401</x:v>
+        <x:v>7.222007</x:v>
       </x:c>
       <x:c r="G3" s="52" t="n">
         <x:v>0.165182</x:v>
@@ -4236,11 +4236,11 @@
         <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0826/2026082600680.pdf</x:v>
       </x:c>
       <x:c r="M3" s="47" t="str">
-        <x:v>Closest listed foundation-model peer; public-market LTM multiple is shown separately from private transaction references. Price refreshed to 2026-10-23; share-count and FX basis carried forward from 2026-08-31.</x:v>
+        <x:v>Closest listed foundation-model peer; public-market LTM multiple is shown separately from private transaction references. Price refreshed to 2026-10-30; share-count and FX basis carried forward from 2026-08-31.</x:v>
       </x:c>
       <x:c r="N3" s="56" t="n">
         <x:f>F3/G3</x:f>
-        <x:v>50.85031811572327</x:v>
+        <x:v>43.721513239941395</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
@@ -4389,13 +4389,13 @@
         <x:v>hk_adjacent</x:v>
       </x:c>
       <x:c r="D7" s="48" t="str">
-        <x:v>2026-10-23</x:v>
+        <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="E7" s="49" t="str">
         <x:v>implied total equity value</x:v>
       </x:c>
       <x:c r="F7" s="53" t="n">
-        <x:v>42.35914805555556</x:v>
+        <x:v>40.35074</x:v>
       </x:c>
       <x:c r="G7" s="53" t="n">
         <x:v>5.567388</x:v>
@@ -4410,17 +4410,17 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K7" s="49" t="str">
-        <x:v>https://query1.finance.yahoo.com/v8/finance/chart/0020.HK?period1=1788134400&amp;period2=1792800000&amp;interval=1d</x:v>
+        <x:v>https://query1.finance.yahoo.com/v8/finance/chart/0020.HK?period1=1792713600&amp;period2=1793404800&amp;interval=1d</x:v>
       </x:c>
       <x:c r="L7" s="49" t="str">
         <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0826/2026082600408.pdf</x:v>
       </x:c>
       <x:c r="M7" s="49" t="str">
-        <x:v>Adjacent Hong Kong AI platform; mixed computer-vision generative-AI and solution revenue makes it contextual only. Price refreshed to 2026-10-23; August share-count and FX basis retained, not a newly verified market capitalization.</x:v>
+        <x:v>Adjacent Hong Kong AI platform; mixed computer-vision generative-AI and solution revenue makes it contextual only. Price refreshed to 2026-10-30; August share-count and FX basis retained, not a newly verified market capitalization.</x:v>
       </x:c>
       <x:c r="N7" s="57" t="n">
         <x:f>F7/G7</x:f>
-        <x:v>7.608441886133238</x:v>
+        <x:v>7.247696765520923</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
@@ -4434,13 +4434,13 @@
         <x:v>hk_adjacent</x:v>
       </x:c>
       <x:c r="D8" s="48" t="str">
-        <x:v>2026-10-23</x:v>
+        <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="E8" s="49" t="str">
         <x:v>implied total equity value</x:v>
       </x:c>
       <x:c r="F8" s="53" t="n">
-        <x:v>10.6098136124197</x:v>
+        <x:v>10.42672</x:v>
       </x:c>
       <x:c r="G8" s="53" t="n">
         <x:v>8.274083</x:v>
@@ -4455,17 +4455,17 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K8" s="49" t="str">
-        <x:v>https://query1.finance.yahoo.com/v8/finance/chart/6682.HK?period1=1788134400&amp;period2=1792800000&amp;interval=1d</x:v>
+        <x:v>https://query1.finance.yahoo.com/v8/finance/chart/6682.HK?period1=1792713600&amp;period2=1793404800&amp;interval=1d</x:v>
       </x:c>
       <x:c r="L8" s="49" t="str">
         <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0820/2026082000357.pdf</x:v>
       </x:c>
       <x:c r="M8" s="49" t="str">
-        <x:v>Enterprise AI platform and agentic services with a different revenue and margin mix; contextual only. Price refreshed to 2026-10-23; August share-count and FX basis retained, not a newly verified market capitalization.</x:v>
+        <x:v>Enterprise AI platform and agentic services with a different revenue and margin mix; contextual only. Price refreshed to 2026-10-30; August share-count and FX basis retained, not a newly verified market capitalization.</x:v>
       </x:c>
       <x:c r="N8" s="57" t="n">
         <x:f>F8/G8</x:f>
-        <x:v>1.2822948008159576</x:v>
+        <x:v>1.2601662323184335</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
@@ -4479,13 +4479,13 @@
         <x:v>hk_adjacent</x:v>
       </x:c>
       <x:c r="D9" s="48" t="str">
-        <x:v>2026-10-23</x:v>
+        <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="E9" s="49" t="str">
         <x:v>implied total equity value</x:v>
       </x:c>
       <x:c r="F9" s="53" t="n">
-        <x:v>8.917234091860463</x:v>
+        <x:v>7.845959</x:v>
       </x:c>
       <x:c r="G9" s="53" t="n">
         <x:v>0.459773</x:v>
@@ -4506,11 +4506,11 @@
         <x:v>https://www1.hkexnews.hk/listedco/listconews/sehk/2026/0825/2026082500959.pdf</x:v>
       </x:c>
       <x:c r="M9" s="49" t="str">
-        <x:v>Decision-intelligence and project-delivery model with a short trading history; contextual only. Price refreshed to 2026-10-23; share-count and FX basis carried forward from 2026-08-31.</x:v>
+        <x:v>Decision-intelligence and project-delivery model with a short trading history; contextual only. Price refreshed to 2026-10-30; share-count and FX basis carried forward from 2026-08-31.</x:v>
       </x:c>
       <x:c r="N9" s="57" t="n">
         <x:f>F9/G9</x:f>
-        <x:v>19.39486244703465</x:v>
+        <x:v>17.06485374304276</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -4524,13 +4524,13 @@
         <x:v>commercialization_reference</x:v>
       </x:c>
       <x:c r="D10" s="32" t="str">
-        <x:v>2026-10-23</x:v>
+        <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="E10" s="50" t="str">
         <x:v>public market equity value</x:v>
       </x:c>
       <x:c r="F10" s="54" t="n">
-        <x:v>472.7745328725219</x:v>
+        <x:v>442.4016240697266</x:v>
       </x:c>
       <x:c r="G10" s="54" t="n">
         <x:v>4.475446</x:v>
@@ -4545,17 +4545,17 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K10" s="50" t="str">
-        <x:v>https://query1.finance.yahoo.com/v8/finance/chart/PLTR?period1=1788134400&amp;period2=1792800000&amp;interval=1d</x:v>
+        <x:v>https://query1.finance.yahoo.com/v8/finance/chart/PLTR?period1=1793318400&amp;period2=1793404800&amp;interval=1d</x:v>
       </x:c>
       <x:c r="L10" s="50" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1321655/000132165526000011/pltr-20251231.htm</x:v>
       </x:c>
       <x:c r="M10" s="50" t="str">
-        <x:v>Mature AI software commercialization reference; not a frontier-model laboratory. Price refreshed to 2026-10-23; August share-count and FX basis retained, not a newly verified market capitalization.</x:v>
+        <x:v>Mature AI software commercialization reference; not a frontier-model laboratory. Price refreshed to 2026-10-30; August share-count and FX basis retained, not a newly verified market capitalization.</x:v>
       </x:c>
       <x:c r="N10" s="58" t="n">
         <x:f>F10/G10</x:f>
-        <x:v>105.6374119746997</x:v>
+        <x:v>98.85084616588529</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -4569,13 +4569,13 @@
         <x:v>commercialization_reference</x:v>
       </x:c>
       <x:c r="D11" s="32" t="str">
-        <x:v>2026-10-23</x:v>
+        <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="E11" s="50" t="str">
         <x:v>public market equity value</x:v>
       </x:c>
       <x:c r="F11" s="54" t="n">
-        <x:v>115.57636588555644</x:v>
+        <x:v>99.59870512601218</x:v>
       </x:c>
       <x:c r="G11" s="54" t="n">
         <x:v>2.1679</x:v>
@@ -4590,17 +4590,17 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K11" s="50" t="str">
-        <x:v>https://query1.finance.yahoo.com/v8/finance/chart/NET?period1=1788134400&amp;period2=1792800000&amp;interval=1d</x:v>
+        <x:v>https://query1.finance.yahoo.com/v8/finance/chart/NET?period1=1793318400&amp;period2=1793404800&amp;interval=1d</x:v>
       </x:c>
       <x:c r="L11" s="50" t="str">
         <x:v>https://www.cloudflare.com/press/press-releases/2026/cloudflare-announces-fourth-quarter-and-fiscal-year-2025-financial-results/</x:v>
       </x:c>
       <x:c r="M11" s="50" t="str">
-        <x:v>Connectivity and inference-infrastructure reference; economics differ from a model laboratory. Price refreshed to 2026-10-23; August share-count and FX basis retained, not a newly verified market capitalization.</x:v>
+        <x:v>Connectivity and inference-infrastructure reference; economics differ from a model laboratory. Price refreshed to 2026-10-30; August share-count and FX basis retained, not a newly verified market capitalization.</x:v>
       </x:c>
       <x:c r="N11" s="58" t="n">
         <x:f>F11/G11</x:f>
-        <x:v>53.31259093387907</x:v>
+        <x:v>45.9424812611339</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
@@ -4614,13 +4614,13 @@
         <x:v>commercialization_reference</x:v>
       </x:c>
       <x:c r="D12" s="32" t="str">
-        <x:v>2026-10-23</x:v>
+        <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="E12" s="50" t="str">
         <x:v>public market equity value</x:v>
       </x:c>
       <x:c r="F12" s="54" t="n">
-        <x:v>112.79423629716236</x:v>
+        <x:v>106.08751224002874</x:v>
       </x:c>
       <x:c r="G12" s="54" t="n">
         <x:v>4.683946</x:v>
@@ -4635,17 +4635,17 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K12" s="50" t="str">
-        <x:v>https://query1.finance.yahoo.com/v8/finance/chart/SNOW?period1=1788134400&amp;period2=1792800000&amp;interval=1d</x:v>
+        <x:v>https://query1.finance.yahoo.com/v8/finance/chart/SNOW?period1=1793318400&amp;period2=1793404800&amp;interval=1d</x:v>
       </x:c>
       <x:c r="L12" s="50" t="str">
         <x:v>https://www.sec.gov/Archives/edgar/data/1640147/000164014726000023/snowflake2026ars.pdf</x:v>
       </x:c>
       <x:c r="M12" s="50" t="str">
-        <x:v>Data-cloud commercialization reference; not a direct foundation-model comparable. Price refreshed to 2026-10-23; August share-count and FX basis retained, not a newly verified market capitalization.</x:v>
+        <x:v>Data-cloud commercialization reference; not a direct foundation-model comparable. Price refreshed to 2026-10-30; August share-count and FX basis retained, not a newly verified market capitalization.</x:v>
       </x:c>
       <x:c r="N12" s="58" t="n">
         <x:f>F12/G12</x:f>
-        <x:v>24.081028324656682</x:v>
+        <x:v>22.649174913636653</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4666,7 +4666,7 @@
         <x:v>Market date</x:v>
       </x:c>
       <x:c r="B1" s="28" t="str">
-        <x:v>2026-10-23</x:v>
+        <x:v>2026-10-30</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -4674,7 +4674,7 @@
         <x:v>Market price (HK$)</x:v>
       </x:c>
       <x:c r="B2" s="14" t="n">
-        <x:v>499</x:v>
+        <x:v>483.6</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4682,7 +4682,7 @@
         <x:v>Market equity value (US$m)</x:v>
       </x:c>
       <x:c r="B3" s="14" t="n">
-        <x:v>31193.1</x:v>
+        <x:v>30230.5</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -4690,7 +4690,7 @@
         <x:v>Market equity value / LTM revenue</x:v>
       </x:c>
       <x:c r="B4" s="14" t="n">
-        <x:v>148.9</x:v>
+        <x:v>144.3</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -4738,7 +4738,7 @@
         <x:v>DCF value as % of market</x:v>
       </x:c>
       <x:c r="B10" s="12" t="n">
-        <x:v>0.2326</x:v>
+        <x:v>0.24</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>